<commit_message>
docs: finalize logical DB design and runtime observability
</commit_message>
<xml_diff>
--- a/docs/22_cera-logical-data-model.xlsx
+++ b/docs/22_cera-logical-data-model.xlsx
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>rev.2.1 (2026-09-17, T-079) · 기준: docs/21 개념 모델 rev.3 (승인) · 짝 문서: docs/22_cera-logical-data-model.md · 사용자 결정 D-1~D-5 전부 CLOSED · 분류(Classification)와 변경 방식(Mutation Policy)은 서로 다른 축이다</t>
+          <t>rev.2.2 최종 정리 (2026-09-18, T-079) · 기준: docs/21 개념 모델 rev.3 (승인) · 짝 문서: docs/22_cera-logical-data-model.md · 사용자 결정 D-1~D-5 전부 CLOSED · 분류(Classification)와 변경 방식(Mutation Policy)은 서로 다른 축이다 · rev.2.2: 기술 운영 표 system_error 추가</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C9" s="9" t="inlineStr"/>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>APPEND_ONLY</t>
+          <t>IMMUTABLE_AFTER_CREATE + CONTROLLED_UPDATE (결과 5컬럼)</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>APPEND_ONLY</t>
+          <t>IMMUTABLE_AFTER_CREATE + CONTROLLED_UPDATE (검토 4컬럼)</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
@@ -2966,84 +2966,82 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
+          <t>system_error</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>시스템·연동 오류 기록</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>EVIDENCE</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>APPEND_ONLY</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>MVP · rev.2.2</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>error_id</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>중요한 시스템/외부 연동 오류를 DB 에서 찾기 위한 기술 운영 표. 업무 개념이 아니다 (docs/23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>09_감사운영</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
           <t>scenario</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>시나리오</t>
         </is>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E63" s="6" t="inlineStr">
         <is>
           <t>SIMULATION_ONLY</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
+      <c r="F63" s="6" t="inlineStr">
         <is>
           <t>CONTROLLED_UPDATE</t>
         </is>
       </c>
-      <c r="G62" s="6" t="inlineStr">
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
-      <c r="H62" s="3" t="inlineStr">
+      <c r="H63" s="3" t="inlineStr">
         <is>
           <t>scenario_id</t>
         </is>
       </c>
-      <c r="I62" s="3" t="inlineStr">
+      <c r="I63" s="3" t="inlineStr">
         <is>
           <t>재생 시나리오. 제품 도메인이 아니다</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t>10_OpenDecisions</t>
-        </is>
-      </c>
-      <c r="C63" s="11" t="inlineStr">
-        <is>
-          <t>exception_case</t>
-        </is>
-      </c>
-      <c r="D63" s="12" t="inlineStr">
-        <is>
-          <t>예외 운영 Case</t>
-        </is>
-      </c>
-      <c r="E63" s="10" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="F63" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G63" s="10" t="inlineStr">
-        <is>
-          <t>CLOSED FOR MVP - 만들지 않는다</t>
-        </is>
-      </c>
-      <c r="H63" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I63" s="12" t="inlineStr">
-        <is>
-          <t>Event -&gt; Risk -&gt; RecoveryRun -&gt; Communication -&gt; Reply -&gt; Re-run 폐쇄 루프에 필수가 아니다. 현재는 파생 조회  [E-36 · L-10 · D-5]</t>
         </is>
       </c>
     </row>
@@ -3060,131 +3058,178 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
+          <t>exception_case</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
+          <t>예외 운영 Case</t>
+        </is>
+      </c>
+      <c r="E64" s="10" t="inlineStr">
+        <is>
+          <t>해당 없음</t>
+        </is>
+      </c>
+      <c r="F64" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G64" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED FOR MVP - 만들지 않는다</t>
+        </is>
+      </c>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I64" s="12" t="inlineStr">
+        <is>
+          <t>Event -&gt; Risk -&gt; RecoveryRun -&gt; Communication -&gt; Reply -&gt; Re-run 폐쇄 루프에 필수가 아니다. 현재는 파생 조회  [E-36 · L-10 · D-5]</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B65" s="10" t="inlineStr">
+        <is>
+          <t>10_OpenDecisions</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
           <t>operational_plan_batch</t>
         </is>
       </c>
-      <c r="D64" s="12" t="inlineStr">
+      <c r="D65" s="12" t="inlineStr">
         <is>
           <t>계획 업로드 묶음</t>
         </is>
       </c>
-      <c r="E64" s="10" t="inlineStr">
+      <c r="E65" s="10" t="inlineStr">
         <is>
           <t>해당 없음</t>
         </is>
       </c>
-      <c r="F64" s="10" t="inlineStr">
+      <c r="F65" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G64" s="10" t="inlineStr">
+      <c r="G65" s="10" t="inlineStr">
         <is>
           <t>CLOSED - 만들지 않는다</t>
         </is>
       </c>
-      <c r="H64" s="12" t="inlineStr">
+      <c r="H65" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I64" s="12" t="inlineStr">
+      <c r="I65" s="12" t="inlineStr">
         <is>
           <t>raw_input 1행이 이미 업로드 1건이고 그 배치의 plan.* 사건이 같은 raw_input_id 를 공유한다  [E-35 · L-9 · D-4]</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="4" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>만들지 않은 것</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>이유</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>truck (개별 차량)</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>MVP 기능이 풀 + 슬롯별 가용량으로 성립한다 (E-39, Q-57)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Money</t>
+          <t>truck (개별 차량)</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>값 객체. cost_line_item 의 금액 컬럼 묶음 (Q-58)</t>
+          <t>MVP 기능이 풀 + 슬롯별 가용량으로 성립한다 (E-39, Q-57)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>phase / container_phase</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>파생. 원본으로 저장하지 않는다 (안티패턴 1)</t>
+          <t>값 객체. cost_line_item 의 금액 컬럼 묶음 (Q-58)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>slot_pool</t>
+          <t>phase / container_phase</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>터미널의 자원 단위. 슬롯 가용은 사실</t>
+          <t>파생. 원본으로 저장하지 않는다 (안티패턴 1)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>destination / carrier</t>
+          <t>slot_pool</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>관계에 붙은 역할. 별도 테이블 아님</t>
+          <t>터미널의 자원 단위. 슬롯 가용은 사실</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>activity_timeline</t>
+          <t>destination / carrier</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>다섯 원본을 합친 조회 뷰</t>
+          <t>관계에 붙은 역할. 별도 테이블 아님</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
+          <t>activity_timeline</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>다섯 원본을 합친 조회 뷰</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
           <t>code_group / code_value</t>
         </is>
       </c>
-      <c r="B73" s="3" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>코드 테이블은 물리 설계에서 형태를 정한다 (18절)</t>
         </is>
@@ -3201,7 +3246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S34"/>
+  <dimension ref="A1:U44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3220,6 +3265,11 @@
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4022,7 +4072,7 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>scenario</t>
+          <t>system_error</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -4032,7 +4082,7 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>시나리오</t>
+          <t>시스템·연동 오류 기록</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -4042,7 +4092,7 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>SIMULATION_ONLY</t>
+          <t>EVIDENCE</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
@@ -4052,7 +4102,7 @@
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>MVP · rev.2.2</t>
         </is>
       </c>
       <c r="J27" s="8" t="inlineStr">
@@ -4062,7 +4112,7 @@
       </c>
       <c r="K27" s="9" t="inlineStr">
         <is>
-          <t>CONTROLLED_UPDATE</t>
+          <t>APPEND_ONLY</t>
         </is>
       </c>
     </row>
@@ -4074,7 +4124,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>재생 시나리오. 제품 도메인이 아니다</t>
+          <t>CERA 안이나 외부 시스템 호출에서 난 중요한 기술 오류를 DB 에서 찾기 위한 기술 운영(관측성) 표. 업무 도메인 개념이 아니다 (docs/21 밖, 행동 규칙 정본 docs/23)</t>
         </is>
       </c>
     </row>
@@ -4086,7 +4136,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>시뮬레이션 전용 테이블을 따로 만들지 않는다. 같은 테이블 + is_simulated + scenario_id</t>
+          <t>event(현실 사실) · audit_log(누가 무엇을 했나) · send_attempt(이 시도가 어떻게 끝났나)와 다르다. 모든 로그를 넣지 않는다 - 중요한 ERROR·외부 연동 실패·예상 밖 5xx·작업 실패만. 비밀값·토큰·메일 본문·전체 스택 트레이스 금지(raw_log_ref 참조만). 행을 고치지 않는다 - 대응 이력 표는 만들지 않았다</t>
         </is>
       </c>
     </row>
@@ -4098,37 +4148,102 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>시나리오 id</t>
+          <t>오류 id</t>
         </is>
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>시나리오명</t>
+          <t>발생 시각</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>서비스</t>
         </is>
       </c>
       <c r="E30" s="16" t="inlineStr">
         <is>
-          <t>데이터 팩 참조</t>
+          <t>구성요소</t>
         </is>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
-          <t>기준 시각</t>
+          <t>작업</t>
         </is>
       </c>
       <c r="G30" s="16" t="inlineStr">
         <is>
-          <t>생성 시각</t>
+          <t>경계</t>
         </is>
       </c>
       <c r="H30" s="16" t="inlineStr">
         <is>
-          <t>활성</t>
+          <t>오류 분류</t>
+        </is>
+      </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>오류 코드</t>
+        </is>
+      </c>
+      <c r="J30" s="16" t="inlineStr">
+        <is>
+          <t>안전한 메시지</t>
+        </is>
+      </c>
+      <c r="K30" s="16" t="inlineStr">
+        <is>
+          <t>예외 종류</t>
+        </is>
+      </c>
+      <c r="L30" s="16" t="inlineStr">
+        <is>
+          <t>요청 id</t>
+        </is>
+      </c>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
+          <t>추적 id</t>
+        </is>
+      </c>
+      <c r="N30" s="16" t="inlineStr">
+        <is>
+          <t>대상 외부 시스템</t>
+        </is>
+      </c>
+      <c r="O30" s="16" t="inlineStr">
+        <is>
+          <t>HTTP 상태</t>
+        </is>
+      </c>
+      <c r="P30" s="16" t="inlineStr">
+        <is>
+          <t>재시도 가능</t>
+        </is>
+      </c>
+      <c r="Q30" s="16" t="inlineStr">
+        <is>
+          <t>관련 개체 종류</t>
+        </is>
+      </c>
+      <c r="R30" s="16" t="inlineStr">
+        <is>
+          <t>관련 개체 id</t>
+        </is>
+      </c>
+      <c r="S30" s="16" t="inlineStr">
+        <is>
+          <t>로그 참조</t>
+        </is>
+      </c>
+      <c r="T30" s="16" t="inlineStr">
+        <is>
+          <t>시뮬레이션</t>
+        </is>
+      </c>
+      <c r="U30" s="16" t="inlineStr">
+        <is>
+          <t>시나리오</t>
         </is>
       </c>
     </row>
@@ -4140,37 +4255,102 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
+          <t>error_id</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>occurred_at</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>service_name</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>component_name</t>
+        </is>
+      </c>
+      <c r="F31" s="19" t="inlineStr">
+        <is>
+          <t>operation_name</t>
+        </is>
+      </c>
+      <c r="G31" s="19" t="inlineStr">
+        <is>
+          <t>error_boundary</t>
+        </is>
+      </c>
+      <c r="H31" s="19" t="inlineStr">
+        <is>
+          <t>error_category</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>error_code</t>
+        </is>
+      </c>
+      <c r="J31" s="19" t="inlineStr">
+        <is>
+          <t>safe_error_message</t>
+        </is>
+      </c>
+      <c r="K31" s="19" t="inlineStr">
+        <is>
+          <t>exception_type</t>
+        </is>
+      </c>
+      <c r="L31" s="19" t="inlineStr">
+        <is>
+          <t>request_id</t>
+        </is>
+      </c>
+      <c r="M31" s="19" t="inlineStr">
+        <is>
+          <t>trace_id</t>
+        </is>
+      </c>
+      <c r="N31" s="19" t="inlineStr">
+        <is>
+          <t>target_system</t>
+        </is>
+      </c>
+      <c r="O31" s="19" t="inlineStr">
+        <is>
+          <t>http_status</t>
+        </is>
+      </c>
+      <c r="P31" s="19" t="inlineStr">
+        <is>
+          <t>retryable</t>
+        </is>
+      </c>
+      <c r="Q31" s="19" t="inlineStr">
+        <is>
+          <t>related_entity_type</t>
+        </is>
+      </c>
+      <c r="R31" s="19" t="inlineStr">
+        <is>
+          <t>related_entity_id</t>
+        </is>
+      </c>
+      <c r="S31" s="19" t="inlineStr">
+        <is>
+          <t>raw_log_ref</t>
+        </is>
+      </c>
+      <c r="T31" s="19" t="inlineStr">
+        <is>
+          <t>is_simulated</t>
+        </is>
+      </c>
+      <c r="U31" s="20" t="inlineStr">
+        <is>
           <t>scenario_id</t>
-        </is>
-      </c>
-      <c r="C31" s="19" t="inlineStr">
-        <is>
-          <t>scenario_name</t>
-        </is>
-      </c>
-      <c r="D31" s="19" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="E31" s="19" t="inlineStr">
-        <is>
-          <t>data_pack_ref</t>
-        </is>
-      </c>
-      <c r="F31" s="19" t="inlineStr">
-        <is>
-          <t>as_of_base</t>
-        </is>
-      </c>
-      <c r="G31" s="19" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="H31" s="19" t="inlineStr">
-        <is>
-          <t>is_active</t>
         </is>
       </c>
     </row>
@@ -4182,37 +4362,102 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>STRING(30)</t>
+          <t>STRING(40)</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
+          <t>TIMESTAMP_TZ</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>STRING(60)</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
           <t>STRING(100)</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>STRING(100)</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>CODE</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>CODE</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>STRING(60)</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>STRING(500)</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>STRING(200)</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>STRING(64)</t>
+        </is>
+      </c>
+      <c r="M32" s="6" t="inlineStr">
+        <is>
+          <t>STRING(64)</t>
+        </is>
+      </c>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>CODE</t>
+        </is>
+      </c>
+      <c r="O32" s="6" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="P32" s="6" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="Q32" s="6" t="inlineStr">
+        <is>
+          <t>CODE</t>
+        </is>
+      </c>
+      <c r="R32" s="6" t="inlineStr">
+        <is>
+          <t>STRING(40)</t>
+        </is>
+      </c>
+      <c r="S32" s="6" t="inlineStr">
         <is>
           <t>STRING(300)</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>STRING(300)</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>TIMESTAMP_TZ</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>TIMESTAMP_TZ</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="T32" s="6" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="U32" s="6" t="inlineStr">
+        <is>
+          <t>REF(scenario)</t>
         </is>
       </c>
     </row>
@@ -4234,27 +4479,92 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>API_REQUEST / INTEGRATION / BACKGROUND_JOB</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL / 값 목록 미확정 (Q-66)</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL / 정규화 코드</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL / 비밀값·본문·스택 금지</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
           <t>NULL 허용</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="L33" s="3" t="inlineStr">
         <is>
           <t>NULL 허용</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용 / 업무 correlation_id 와 다름</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용 / GMAIL / UNIPASS / DATA_GO_KR / LLM_PROVIDER …</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용</t>
+        </is>
+      </c>
+      <c r="P33" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL / 분류 규칙이 판정</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용 / 다형 참조</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용 / DB FK 없음</t>
+        </is>
+      </c>
+      <c r="S33" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용 / 외부 로그 위치만</t>
+        </is>
+      </c>
+      <c r="T33" s="3" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
+      <c r="U33" s="3" t="inlineStr">
+        <is>
+          <t>is_simulated=true 일 때만</t>
         </is>
       </c>
     </row>
@@ -4266,35 +4576,488 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
+          <t>ERR-000001</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T10:05+09:00</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>back-worker</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>channels.gmail</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>send_message</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>INTEGRATION</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>EXTERNAL_SERVER_ERROR</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>GMAIL_SERVER_ERROR</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Gmail send returned 503</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>(예외 클래스명)</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>req-(예시)</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>trc-(예시)</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>GMAIL</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>503</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>SEND_ATTEMPT</t>
+        </is>
+      </c>
+      <c r="R34" s="3" t="inlineStr">
+        <is>
+          <t>SND-0001</t>
+        </is>
+      </c>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>log://(예시)</t>
+        </is>
+      </c>
+      <c r="T34" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="U34" s="3" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>예시 2</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>ERR-000002</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T10:40+09:00</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>back-api</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>extraction.email</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>parse_reply</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>INTEGRATION</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>EXTERNAL_RESPONSE_INVALID</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>EXTERNAL_RESPONSE_INVALID</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>LLM 응답이 추출 스키마와 맞지 않음</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>(예외 클래스명)</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>req-(예시)</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>trc-(예시)</t>
+        </is>
+      </c>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>LLM_PROVIDER</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="n"/>
+      <c r="P35" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>EXTRACTION</t>
+        </is>
+      </c>
+      <c r="R35" s="3" t="inlineStr">
+        <is>
+          <t>EXT-0009</t>
+        </is>
+      </c>
+      <c r="S35" s="3" t="inlineStr">
+        <is>
+          <t>log://(예시)</t>
+        </is>
+      </c>
+      <c r="T35" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="U35" s="3" t="inlineStr">
+        <is>
           <t>SCN-BUSAN-WH-01</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>영문 테이블명</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>한글 테이블명</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>시나리오</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>분류</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>SIMULATION_ONLY</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>단계</t>
+        </is>
+      </c>
+      <c r="I37" s="9" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>변경 방식</t>
+        </is>
+      </c>
+      <c r="K37" s="9" t="inlineStr">
+        <is>
+          <t>CONTROLLED_UPDATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>재생 시나리오. 제품 도메인이 아니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>주의</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>시뮬레이션 전용 테이블을 따로 만들지 않는다. 같은 테이블 + is_simulated + scenario_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>한글 필드명</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>시나리오 id</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>시나리오명</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>데이터 팩 참조</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>기준 시각</t>
+        </is>
+      </c>
+      <c r="G40" s="16" t="inlineStr">
+        <is>
+          <t>생성 시각</t>
+        </is>
+      </c>
+      <c r="H40" s="16" t="inlineStr">
+        <is>
+          <t>활성</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>영문 필드명</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>scenario_id</t>
+        </is>
+      </c>
+      <c r="C41" s="19" t="inlineStr">
+        <is>
+          <t>scenario_name</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E41" s="19" t="inlineStr">
+        <is>
+          <t>data_pack_ref</t>
+        </is>
+      </c>
+      <c r="F41" s="19" t="inlineStr">
+        <is>
+          <t>as_of_base</t>
+        </is>
+      </c>
+      <c r="G41" s="19" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="H41" s="19" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>타입</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>STRING(30)</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>STRING(100)</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>STRING(300)</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>STRING(300)</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>TIMESTAMP_TZ</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>TIMESTAMP_TZ</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>예시 1</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>SCN-BUSAN-WH-01</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>부산 창고 수용량 예외 30대</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>Prototype 기준 시나리오</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>data/scenarios/busan-wh-capacity-01/</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>2026-09-18T06:00+09:00</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>2026-09-15T00:00+09:00</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H44" s="3" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -4311,7 +5074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4325,7 +5088,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>사용자 결정 결과 · 열린 질문 판정 (rev.2)</t>
+          <t>사용자 결정 결과 · 열린 질문 판정 (rev.2.2 최종 정리)</t>
         </is>
       </c>
     </row>
@@ -4839,7 +5602,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>question_item 이 target_entity_*/target_fact_key 를 갖고 ask_id 로 단건 조회</t>
+          <t>question_item 이 target_entity_type/id · target_fact_key · target_applicability_scope_type/ref(rev.2.1) 를 질문 생성 시 확정하고 ask_id 로 단건 조회. 개체·사실 키·적용 범위가 모두 그 행에서 나오며 LLM 은 범위를 만지지 않는다</t>
         </is>
       </c>
     </row>
@@ -5195,101 +5958,137 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="23" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Q-66</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>system_error 의 오류 분류·코드 값 목록</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>OPEN - rev.2.2 신규</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>예시(GMAIL_TIMEOUT · GMAIL_RATE_LIMITED · GMAIL_AUTH_EXPIRED · EXTERNAL_RESPONSE_INVALID)만 적었다. 전체 목록은 T-069 구현 계획·구현에서 정한다 (docs/23 6절)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="23" t="inlineStr">
         <is>
           <t>[4] 이번 단계에서 정하지 않는 것</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>DB 제품 (PostgreSQL / MySQL / SQLite)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>ORM</t>
+          <t>DB 제품 (PostgreSQL / MySQL / SQLite)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>실제 CREATE TABLE SQL / 마이그레이션</t>
+          <t>ORM</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>인덱스·파티션·복제</t>
+          <t>실제 CREATE TABLE SQL / 마이그레이션</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>API endpoint</t>
+          <t>인덱스·파티션·복제</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>LLM 공급자·모델</t>
+          <t>API endpoint</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>솔버와 그 내부 표현</t>
+          <t>LLM 공급자·모델</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>위험·신선도·근거 강도의 실제 임계값</t>
+          <t>솔버와 그 내부 표현</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>plan_decision.decision_type 의 값 목록</t>
+          <t>위험·신선도·근거 강도의 실제 임계값</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>applicability_scope_type 값 목록 (L-14)</t>
+          <t>plan_decision.decision_type 의 값 목록</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>복구 맥락 식별자 (L-13)</t>
+          <t>applicability_scope_type 값 목록 (L-14)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>bl 의 실제 UNIQUE 제약 (L-16)</t>
+          <t>복구 맥락 식별자 (L-13)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
+          <t>bl 의 실제 UNIQUE 제약 (L-16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
           <t>적용 범위 사이의 우선순위 규칙 (L-14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>system_error 오류 분류·코드 값 목록 (Q-66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Backend 언어·프레임워크 (ADR-031 Proposed, docs/23)</t>
         </is>
       </c>
     </row>
@@ -11039,7 +11838,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>rev.2: source_tier 제거(근거 강도는 계산 결과 -&gt; canonical_fact). 원천 축만 남긴다. 적용 범위(scope)와 유효 기간(validity)은 다른 축이다. 예시 3 = 운영자의 '이번 건만 0원'</t>
+          <t>rev.2: source_tier 제거(근거 강도는 계산 결과 -&gt; canonical_fact). 원천 축만 남긴다. 적용 범위(scope)와 유효 기간(validity)은 다른 축이다. 예시 3 = 운영자의 '이번 건만 0원' / rev.2.2: 복구 맥락 참조는 자리표시자 &lt;RECOVERY_CONTEXT_REF&gt; 로 적는다 - 별도 RecoveryContext 표도, recovery_run id 라는 뜻도 아니다. 식별 방식은 L-13 이 정한다</t>
         </is>
       </c>
     </row>
@@ -11859,7 +12658,7 @@
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>&lt;RECOVERY_CONTEXT_REF&gt;</t>
         </is>
       </c>
       <c r="O28" s="3" t="inlineStr">
@@ -13100,7 +13899,7 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>&lt;RECOVERY_CONTEXT_REF&gt;</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -14386,7 +15185,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>&lt;RECOVERY_CONTEXT_REF&gt;</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr"/>
@@ -17791,7 +18590,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>&lt;RECOVERY_CONTEXT_REF&gt;</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -18205,7 +19004,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>&lt;RECOVERY_CONTEXT_REF&gt;</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
@@ -18290,7 +19089,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>사실이 없어 마스터 기본값으로 계산했다면 그 값을 남긴다. 마스터는 수정 가능하므로 나중에 고치면 과거 실행이 재현되지 않는다. tariff_rule 은 불변 판이라 id 참조로 충분하다</t>
+          <t>사실이 없어 마스터 기본값으로 계산했다면 그 값을 남긴다. 마스터는 수정 가능하므로 나중에 고치면 과거 실행이 재현되지 않는다. tariff_rule 은 불변 판이라 id 참조로 충분하다 / rev.2.2: value_path 는 PK 일부라 NOT NULL. 예시 2 의 &lt;WHOLE_ROW&gt; 는 '행 전체' 를 뜻하는 자리표시자이고 실제 문자열은 T-080 에서 정한다</t>
         </is>
       </c>
     </row>
@@ -18478,7 +19277,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>NULL 허용 / 컬럼 이름</t>
+          <t>NOT NULL / MASTER_DEFAULT = 컬럼 경로 · 행/판 전체 = 논리적 '전체' 표시 (물리 문자열은 T-080)</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -18572,7 +19371,11 @@
           <t>TRF-0001</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr"/>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>&lt;WHOLE_ROW&gt;</t>
+        </is>
+      </c>
       <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr">
@@ -20403,7 +21206,7 @@
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>&lt;RECOVERY_CONTEXT_REF&gt;</t>
         </is>
       </c>
       <c r="L84" s="3" t="inlineStr">
@@ -20473,7 +21276,7 @@
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>&lt;RECOVERY_CONTEXT_REF&gt;</t>
         </is>
       </c>
       <c r="L85" s="3" t="inlineStr">
@@ -20547,7 +21350,7 @@
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>&lt;RECOVERY_CONTEXT_REF&gt;</t>
         </is>
       </c>
       <c r="L86" s="3" t="inlineStr"/>
@@ -23563,7 +24366,7 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>&lt;RECOVERY_CONTEXT_REF&gt;</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
@@ -24960,7 +25763,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>rev.2.1: 행 종류별 필수 컬럼이 다르다. APPROVED = 내용·수신자·지문·구조화 값 사본 필수. REJECTED/REVISION_REQUESTED = 사유 필수, 내용 사본은 선택. REVOKED/INVALIDATED = 대상 + 사유 종류만 필수이고 승인 사본을 새로 요구하지 않는다. 만료는 expires_at(만들 때 정함). 어떤 행도 UPDATE 하지 않는다</t>
+          <t>rev.2.1·rev.2.2: 행 종류별 필수 컬럼이 다르다. APPROVED = approved_content_hash · approved_to_address_id 필수 + 메시지에 값이 있는 범위에서 제목·본문·구조화 값 사본 필수. REJECTED/REVISION_REQUESTED = reason 필수, 사본 조건을 적용하지 않는다. REVOKED/INVALIDATED = invalidates_approval_id + invalidation_cause 필수, 새 지문·사본 불필요, 대상은 같은 message_id 의 기존 APPROVED. 만료는 expires_at(만들 때 정함). 어떤 행도 UPDATE 하지 않는다</t>
         </is>
       </c>
     </row>
@@ -25243,17 +26046,17 @@
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>APPROVED 면 필수 / 사본</t>
+          <t>APPROVED 이고 원 메시지에 값이 있으면 필수 / 사본 (값이 없는 메시지에 빈 사본을 요구하지 않는다)</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>APPROVED 면 필수 / 사본</t>
+          <t>APPROVED 이고 원 메시지에 값이 있으면 필수 / 사본 (값이 없는 메시지에 빈 사본을 요구하지 않는다)</t>
         </is>
       </c>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t>NULL 허용</t>
+          <t>NULL 허용 / 계획 기반 메시지의 APPROVED 면 필수</t>
         </is>
       </c>
       <c r="M63" s="3" t="inlineStr">
@@ -25268,7 +26071,7 @@
       </c>
       <c r="O63" s="3" t="inlineStr">
         <is>
-          <t>NULL 허용</t>
+          <t>REJECTED·REVISION_REQUESTED 면 필수 / 무효화일 때 권장</t>
         </is>
       </c>
     </row>
@@ -25798,7 +26601,7 @@
       </c>
       <c r="K77" s="9" t="inlineStr">
         <is>
-          <t>APPEND_ONLY</t>
+          <t>IMMUTABLE_AFTER_CREATE + CONTROLLED_UPDATE (결과 5컬럼)</t>
         </is>
       </c>
     </row>
@@ -25822,7 +26625,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>rev.2.1: 지문 비교 대상이 종류별로 다르다. BUSINESS = 유효한 승인의 approved_content_hash, CONTACT_VERIFICATION = 그 메시지 자신의 content_hash. 어느 쪽도 '작성한 내용 != 보낸 내용' 은 허용하지 않는다. approval_id 는 메시지 종류에 따른 조건부 필수. UNKNOWN 을 성공·실패로 접지 않는다</t>
+          <t>rev.2.2: 식별·요청 9컬럼(send_attempt_id·message_id·approval_id·attempt_no·idempotency_key·channel_connection_id·sent_content_hash·started_at·is_simulated)은 불변. 결과 5컬럼(finished_at·result·error_code·error_message·provider_message_id)만 호출 뒤 한 번 기록. 재시도는 새 행. 기술 오류 상세는 system_error. rev.2.1: 지문 비교 대상이 종류별로 다르다. BUSINESS = 유효한 승인의 approved_content_hash, CONTACT_VERIFICATION = 그 메시지 자신의 content_hash. UNKNOWN 을 성공·실패로 접지 않는다</t>
         </is>
       </c>
     </row>
@@ -26100,17 +26903,17 @@
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>NOT NULL / 외부 호출 전에 기록</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>NULL 허용</t>
+          <t>NULL 허용 / 결과 기록 때 한 번</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>SUCCESS / RETRYABLE_FAILURE / PERMANENT_FAILURE / UNKNOWN</t>
+          <t>NULL = 결과 기록 전 / SUCCESS / RETRYABLE_FAILURE / PERMANENT_FAILURE / UNKNOWN - 한 번만</t>
         </is>
       </c>
       <c r="L83" s="3" t="inlineStr">
@@ -26668,7 +27471,7 @@
       </c>
       <c r="K97" s="9" t="inlineStr">
         <is>
-          <t>APPEND_ONLY</t>
+          <t>IMMUTABLE_AFTER_CREATE + CONTROLLED_UPDATE (검토 4컬럼)</t>
         </is>
       </c>
     </row>
@@ -26692,7 +27495,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>신원·권한·근거 강도·상태 확정·숫자는 여기서 정하지 않는다 (ADR-026·029)</t>
+          <t>rev.2.2: 추출 결과(후보 값·인용·모델 판·프롬프트 판 등)는 불변. 검토 4컬럼(review_status·reviewed_by_actor_id·reviewed_at·created_event_id)만 PENDING -&gt; ACCEPTED/REJECTED/SUPERSEDED 한 방향 한 번. 신원·권한·근거 강도·상태 확정·숫자는 여기서 정하지 않는다 (ADR-026·029)</t>
         </is>
       </c>
     </row>
@@ -27020,7 +27823,7 @@
       </c>
       <c r="M103" s="3" t="inlineStr">
         <is>
-          <t>PENDING / ACCEPTED / REJECTED / SUPERSEDED</t>
+          <t>PENDING / ACCEPTED / REJECTED / SUPERSEDED - 한 방향 한 번</t>
         </is>
       </c>
       <c r="N103" s="3" t="inlineStr">
@@ -27035,7 +27838,7 @@
       </c>
       <c r="P103" s="3" t="inlineStr">
         <is>
-          <t>NULL 허용</t>
+          <t>NULL 허용 / ACCEPTED 면 필수</t>
         </is>
       </c>
       <c r="Q103" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: close Q-44 mail time rule and Q-45 record/content retention
T-069 전에 필요했던 사용자 결정 Q-44 · Q-45 를 정본에 반영하고
Q-45 에 필요한 최소 논리 구조만 보완한다. 새 표 없음.
docs/21 변경 없음.

Q-44 (CLOSED)
- 메일 source_recorded_at: Date 헤더가 있고 파싱되고 채널 수신 시각
  (Gmail internalDate)보다 미래가 아니면 Date, 아니면 채널 수신 시각
  + date_header_rejected · 사유. 과거 Date 는 허용
- 원래 두 시각과 선택 결과는 event.payload 에 보존 (docs/22 11.2e)

Q-45 (구조 CLOSED / 기간 OPEN)
- 기록과 내용 분리: 행 삭제 != 내용 파기 (docs/22 29절, ADR-032)
- 내용 컬럼을 참조 + 지문으로: message_content_ref,
  approved_content_ref, source_quote_ref/_hash,
  conditions_content_ref/_hash, raw_input.attachment_manifest
- 파기 가능 조건, CONTENT_PURGED 감사(기존 audit_log 컬럼)
- 정상 파기 vs 데이터 손실 구분: 성공한 CONTENT_PURGED 감사가 없는
  내용 부재는 손실(system_error) (I-34)
- 재현성 != 원문 재처리 능력. 보관 기간 숫자는 Pilot 정책

docs/18 F.2 를 rev.2.3 필드명으로 정리.
논리 테이블 52 그대로, 작업표 블록 53 · 컬럼 587, 흐름 검증 64개 PASS.
</commit_message>
<xml_diff>
--- a/docs/22_cera-logical-data-model.xlsx
+++ b/docs/22_cera-logical-data-model.xlsx
@@ -581,7 +581,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>rev.2.3 논리 모델 후속 T-081 DONE (2026-09-21, 사용자 최종 승인). docs/05 4.2 대조로 누락 13건 복구 + ADR-020 상태 차원 복구. 표 +1. 흐름 검증 47개 PASS</t>
+          <t>rev.2.4 Q-44 · Q-45 사용자 결정 반영 (2026-09-21). 메일 근거 시각 규칙 + 기록·내용 분리 보관. 표 수 변화 없음. 흐름 검증 64개 PASS. (rev.2.3 T-081 DONE 위)</t>
         </is>
       </c>
     </row>
@@ -3707,6 +3707,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="8" t="n">
         <v>2</v>
@@ -3782,7 +3783,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>사람의 결정은 plan_decision / message_approval / verification_request_handling 에 남는다. 감사는 그 위의 행위 기록</t>
+          <t>사람의 결정은 plan_decision / message_approval / verification_request_handling 에 남는다. 감사는 그 위의 행위 기록 / rev.2.4 (Q-45): 내용 파기도 감사한다 — action = CONTENT_PURGED, target_type = 내용 범주, target_id = 기록 id, request_context = 보관 정책 판, result. 파기한 내용은 여기에 복사하지 않는다 / 내용 부재는 성공한 CONTENT_PURGED 가 있을 때만 정상 파기. 감사 없는 부재는 데이터 손실(system_error). SUCCESS 는 제거 확인 뒤에만</t>
         </is>
       </c>
     </row>
@@ -5109,7 +5110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5137,7 +5138,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>[1] 사용자 결정 (6건 - D-1~D-5 2026-09-17, C 2026-09-21 전부 CLOSED)</t>
+          <t>[1] 사용자 결정 (8건 - D-1~D-5 2026-09-17, C · Q-44 · Q-45(구조) 2026-09-21 전부 CLOSED)</t>
         </is>
       </c>
     </row>
@@ -5365,631 +5366,651 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Q-44</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>메일 Date 헤더와 채널 수신 시각이 다를 때 source_recorded_at</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>① 대칭 허용 오차  ② 방향별(미래 Date 만 거부)  ③ 항상 internalDate  ④ 항상 Date  ⑤ 비움</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED - ② (2026-09-21 사용자 결정)</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Date 가 채널 수신 시각보다 미래가 아니면 Date. 늦게 도착한 메일을 최신처럼 만들지 않고, 미래 Date 위장을 막는다. 원래 두 시각은 event.payload</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>보통 - 두 시각을 보존했으므로 원문 파기 뒤에도 재판정 가능</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Q-45</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>실제 메일 보관·파기 정책</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>① 기록·내용 분리 + 단계적 파기  ② 무기한  ③ 원문 즉시 파기  ④ Pilot 까지 보류</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>구조 CLOSED - ① (2026-09-21 사용자 결정) / 기간 숫자 OPEN (Pilot 정책)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>행 삭제 ≠ 내용 파기. 내용은 참조 + 지문, 기록은 파기하지 않는다. 새 표 없음 (29절)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>구조: 어려움(처음부터 필요) / 기간 숫자: 쉬움 / 이미 파기한 내용: 되돌릴 수 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>[2] MVP 에서 만들지 않기로 한 테이블</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>영문 테이블명</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>한글</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>근거 항목</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>결정</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>근거</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>다시 여는 조건</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>exception_case</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>예외 운영 Case</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>E-36 · L-10 · D-5</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>CLOSED FOR MVP - 만들지 않는다</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Event -&gt; Risk -&gt; RecoveryRun -&gt; Communication -&gt; Reply -&gt; Re-run 폐쇄 루프에 필수가 아니다. 현재는 파생 조회</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>다시 여는 조건: 담당자 배정 · 예외 건 상태 · 종결 · SLA · Case 단위 협업. 만들 때는 결정적 case_key</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>operational_plan_batch</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>계획 업로드 묶음</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>E-35 · L-9 · D-4</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>CLOSED - 만들지 않는다</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>raw_input 1행이 이미 업로드 1건이고 그 배치의 plan.* 사건이 같은 raw_input_id 를 공유한다</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>다시 여는 조건: 배치 이름 · 상태 · 버전 · 승인 · 묶음 단위 되돌리기/교체</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>[3] 이번 단계에서 판정한 열린 질문</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>번호</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>질문</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>결론</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>스키마 반영</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>Q-54</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>외부 시스템 식별자 저장 구조</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>하이브리드</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>조회 경로 id 는 컬럼(comm_message/comm_thread), 화물·통관 id 는 external_identifier</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>Q-55</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>시설 하위 종류 구조</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>공통 + 1:1 상세</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>facility + facility_warehouse / facility_terminal / facility_odcy</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="19" t="inlineStr">
         <is>
-          <t>Q-58</t>
+          <t>Q-54</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>금액·통화 표현</t>
+          <t>외부 시스템 식별자 저장 구조</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>컬럼 묶음</t>
+          <t>하이브리드</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Money 테이블 없음. amount_krw + original_currency/amount + fx_rate + fx_rate_basis_date</t>
+          <t>조회 경로 id 는 컬럼(comm_message/comm_thread), 화물·통관 id 는 external_identifier</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Q-59</t>
+          <t>Q-55</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>확인 요청 처리 기록의 참조 대상</t>
+          <t>시설 하위 종류 구조</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>결정적 request_key (DB FK 아님)</t>
+          <t>공통 + 1:1 상세</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>rev.2: DB 외래키가 아니라 논리 연결 키. 재료에서 conflict_id 같은 파생 대리키 제거</t>
+          <t>facility + facility_warehouse / facility_terminal / facility_odcy</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>Q-60</t>
+          <t>Q-58</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>CostLineItem 의 귀속</t>
+          <t>금액·통화 표현</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>필수 부모 1개 + 링크 테이블</t>
+          <t>컬럼 묶음</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>cost_result_id 만 NOT NULL. 귀속·근거는 cost_line_link(link_role)</t>
+          <t>Money 테이블 없음. amount_krw + original_currency/amount + fx_rate + fx_rate_basis_date</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>Q-62</t>
+          <t>Q-59</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Actor 구조</t>
+          <t>확인 요청 처리 기록의 참조 대상</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>최소 구성</t>
+          <t>결정적 request_key (DB FK 아님)</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>actor_id / actor_type / display_name / is_active. 인증·권한은 나중</t>
+          <t>rev.2: DB 외래키가 아니라 논리 연결 키. 재료에서 conflict_id 같은 파생 대리키 제거</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>Q-63</t>
+          <t>Q-60</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>fact_key 분해</t>
+          <t>CostLineItem 의 귀속</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>원본은 문자열 유지</t>
+          <t>필수 부모 1개 + 링크 테이블</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>event.fact_key 는 불변 문자열. 파생 canonical_fact 에만 param_* 분해 컬럼</t>
+          <t>cost_result_id 만 NOT NULL. 귀속·근거는 cost_line_link(link_role)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="19" t="inlineStr">
         <is>
-          <t>L-1</t>
+          <t>Q-62</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>회신 값을 원래 질문에 되붙이기</t>
+          <t>Actor 구조</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>질문 생성 시 대상 확정</t>
+          <t>최소 구성</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>question_item 이 target_entity_type/id · target_fact_key · target_applicability_scope_type/ref(rev.2.1) 를 질문 생성 시 확정하고 ask_id 로 단건 조회. 개체·사실 키·적용 범위가 모두 그 행에서 나오며 LLM 은 범위를 만지지 않는다</t>
+          <t>actor_id / actor_type / display_name / is_active. 인증·권한은 나중</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="19" t="inlineStr">
         <is>
-          <t>L-2</t>
+          <t>Q-63</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Container ↔ B/L</t>
+          <t>fact_key 분해</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>연결 테이블</t>
+          <t>원본은 문자열 유지</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>container_bl + PRIMARY 부분 유일 제약 (D-1 CLOSED)</t>
+          <t>event.fact_key 는 불변 문자열. 파생 canonical_fact 에만 param_* 분해 컬럼</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>L-3</t>
+          <t>L-1</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>제안 묶음</t>
+          <t>회신 값을 원래 질문에 되붙이기</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>테이블로 만든다</t>
+          <t>질문 생성 시 대상 확정</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>commercial_offer + item, 분류 EVIDENCE (D-2 CLOSED)</t>
+          <t>question_item 이 target_entity_type/id · target_fact_key · target_applicability_scope_type/ref(rev.2.1) 를 질문 생성 시 확정하고 ask_id 로 단건 조회. 개체·사실 키·적용 범위가 모두 그 행에서 나오며 LLM 은 범위를 만지지 않는다</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>L-3b</t>
+          <t>L-2</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>운영자 입력 요율의 적용 대상·기간</t>
+          <t>Container ↔ B/L</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>범위와 기간을 분리</t>
+          <t>연결 테이블</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>rev.2: valid_from/until(시간) 과 applicability_scope_type/ref(대상) 을 다른 축으로. 기본 RECOVERY_CONTEXT</t>
+          <t>container_bl + PRIMARY 부분 유일 제약 (D-1 CLOSED)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>L-4</t>
+          <t>L-3</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>마스터 값 vs 사실</t>
+          <t>제안 묶음</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>default_ 접두</t>
+          <t>테이블로 만든다</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>마스터에는 평시 기준선만. 그날 값은 사실이 이긴다. 계산에 쓴 기본값은 스냅샷에 얼린다</t>
+          <t>commercial_offer + item, 분류 EVIDENCE (D-2 CLOSED)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="19" t="inlineStr">
         <is>
-          <t>L-5</t>
+          <t>L-3b</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>차량 표현</t>
+          <t>운영자 입력 요율의 적용 대상·기간</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>풀 단위</t>
+          <t>범위와 기간을 분리</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>plan.truck_pool / plan.depart_slot 사실. 개별 차량 없음</t>
+          <t>rev.2: valid_from/until(시간) 과 applicability_scope_type/ref(대상) 을 다른 축으로. 기본 RECOVERY_CONTEXT</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>L-6</t>
+          <t>L-4</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>예외 처리 단위</t>
+          <t>마스터 값 vs 사실</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>L-10 으로 합침</t>
+          <t>default_ 접두</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>D-5 CLOSED FOR MVP</t>
+          <t>마스터에는 평시 기준선만. 그날 값은 사실이 이긴다. 계산에 쓴 기본값은 스냅샷에 얼린다</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>L-7</t>
+          <t>L-5</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>발송 시도</t>
+          <t>차량 표현</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>별도 테이블</t>
+          <t>풀 단위</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>send_attempt. rev.2: 승인은 메시지 종류에 따른 조건부 필수</t>
+          <t>plan.truck_pool / plan.depart_slot 사실. 개별 차량 없음</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>L-8</t>
+          <t>L-6</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>시뮬레이션 분리</t>
+          <t>예외 처리 단위</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>같은 테이블 + 플래그</t>
+          <t>L-10 으로 합침</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>is_simulated + scenario_id, 산출물은 contains_simulated 로 전파</t>
+          <t>D-5 CLOSED FOR MVP</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
         <is>
-          <t>L-9</t>
+          <t>L-7</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>계획 업로드 묶음</t>
+          <t>발송 시도</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>만들지 않는다</t>
+          <t>별도 테이블</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>raw_input 이 배치 출처 (D-4 CLOSED)</t>
+          <t>send_attempt. rev.2: 승인은 메시지 종류에 따른 조건부 필수</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="19" t="inlineStr">
         <is>
-          <t>L-10</t>
+          <t>L-8</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>ExceptionCase</t>
+          <t>시뮬레이션 분리</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>MVP 에서 만들지 않는다</t>
+          <t>같은 테이블 + 플래그</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>파생 조회 (D-5 CLOSED FOR MVP)</t>
+          <t>is_simulated + scenario_id, 산출물은 contains_simulated 로 전파</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>L-11</t>
+          <t>L-9</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>MessageApproval</t>
+          <t>계획 업로드 묶음</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>덧붙이기 + 승인 사본 + 무효화 행</t>
+          <t>만들지 않는다</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>rev.2: 구조화 값까지 얼리고, 취소·만료·계획 교체를 UPDATE 없이 남긴다</t>
+          <t>raw_input 이 배치 출처 (D-4 CLOSED)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="19" t="inlineStr">
         <is>
-          <t>L-12</t>
+          <t>L-10</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>운영자 계획 조건</t>
+          <t>ExceptionCase</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>별도 DECISION_RECORD 테이블</t>
+          <t>MVP 에서 만들지 않는다</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>rev.2: 해제도 action=RELEASE 새 행. 기본 범위는 RECOVERY_CONTEXT. 솔버 표현은 미확정</t>
+          <t>파생 조회 (D-5 CLOSED FOR MVP)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="19" t="inlineStr">
         <is>
-          <t>L-13</t>
+          <t>L-11</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>복구 맥락(Recovery Context)의 식별자</t>
+          <t>MessageApproval</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>OPEN - rev.2 신규</t>
+          <t>덧붙이기 + 승인 사본 + 무효화 행</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>후보: recovery_run 계보의 뿌리 / 최초 계기 사건 / 컨테이너 집합 지문. T-069 에서 답한다</t>
+          <t>rev.2: 구조화 값까지 얼리고, 취소·만료·계획 교체를 UPDATE 없이 남긴다</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t>L-14</t>
+          <t>L-12</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>적용 범위의 값 목록 + 범위 선택 정책</t>
+          <t>운영자 계획 조건</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>OPEN - rev.2 신규 / rev.2.1 확장</t>
+          <t>별도 DECISION_RECORD 테이블</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>① 값 목록 enum 미확정 (기본값이 RECOVERY_CONTEXT 라는 것만 확정) ② 여러 범위가 동시에 적용 가능할 때의 선택 정책도 확정하지 않는다 - CONTRACT/CONTAINER/RECOVERY_CONTEXT 는 서로 다른 축이라 한 줄로 못 세운다. 확정한 것: 범위는 사실 식별자에 포함 · 같은 범위끼리만 Reconciliation · 결정론적 선택 정책이 필요함 · 쓴 범위는 스냅샷에 남음</t>
+          <t>rev.2: 해제도 action=RELEASE 새 행. 기본 범위는 RECOVERY_CONTEXT. 솔버 표현은 미확정</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>L-15</t>
+          <t>L-13</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>message_kind 값 목록</t>
+          <t>복구 맥락(Recovery Context)의 식별자</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -5999,228 +6020,279 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>지금은 BUSINESS / CONTACT_VERIFICATION 둘만. 늘리는 것은 쉽다</t>
+          <t>후보: recovery_run 계보의 뿌리 / 최초 계기 사건 / 컨테이너 집합 지문. T-069 에서 답한다</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>L-16</t>
+          <t>L-14</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>bl 의 업무 유일 제약</t>
+          <t>적용 범위의 값 목록 + 범위 선택 정책</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>OPEN - rev.2 신규</t>
+          <t>OPEN - rev.2 신규 / rev.2.1 확장</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>(bl_type, bl_no, bl_year) 는 후보일 뿐. 번호가 연도 안에서 유일한지 미확인. 실데이터 확인 뒤 물리 설계</t>
+          <t>① 값 목록 enum 미확정 (기본값이 RECOVERY_CONTEXT 라는 것만 확정) ② 여러 범위가 동시에 적용 가능할 때의 선택 정책도 확정하지 않는다 - CONTRACT/CONTAINER/RECOVERY_CONTEXT 는 서로 다른 축이라 한 줄로 못 세운다. 확정한 것: 범위는 사실 식별자에 포함 · 같은 범위끼리만 Reconciliation · 결정론적 선택 정책이 필요함 · 쓴 범위는 스냅샷에 남음</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="19" t="inlineStr">
         <is>
+          <t>L-15</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>message_kind 값 목록</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>OPEN - rev.2 신규</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>지금은 BUSINESS / CONTACT_VERIFICATION 둘만. 늘리는 것은 쉽다</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>L-16</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>bl 의 업무 유일 제약</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>OPEN - rev.2 신규</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>(bl_type, bl_no, bl_year) 는 후보일 뿐. 번호가 연도 안에서 유일한지 미확인. 실데이터 확인 뒤 물리 설계</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
           <t>Q-66</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>system_error 의 오류 분류·코드 값 목록</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>OPEN - rev.2.2 신규</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>예시(GMAIL_TIMEOUT · GMAIL_RATE_LIMITED · GMAIL_AUTH_EXPIRED · EXTERNAL_RESPONSE_INVALID)만 적었다. 전체 목록은 T-069 구현 계획·구현에서 정한다 (docs/23 6절)</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Q-46</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>상대방이 직접 입력한 구조화 값의 Source 모델</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>OPEN - 유지 (rev.2.3 에서 닫지 않았다)</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>source_type 7값은 현재 ADR-020 기준의 정렬이지 영구 확정 enum 이 아니다. HUMAN_UI 로 넣으면 거래처 입력이 CERA 사용자 입력과 같은 강도가 되어 권한 모델이 무너진다. actor_type 축 신설 여부는 권한 모델과 함께 정한다</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Q-34</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>event.payload.change_reason 의 값 목록</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>OPEN - rev.2.3 신규</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>R6 변화 선언 예외 판정의 입력. 값 목록은 T-037 · 인터뷰</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="23" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="23" t="inlineStr">
         <is>
           <t>[4] 이번 단계에서 정하지 않는 것</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>DB 제품 (PostgreSQL / MySQL / SQLite)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>ORM</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>실제 CREATE TABLE SQL / 마이그레이션</t>
+          <t>DB 제품 (PostgreSQL / MySQL / SQLite)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>인덱스·파티션·복제</t>
+          <t>ORM</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>API endpoint</t>
+          <t>실제 CREATE TABLE SQL / 마이그레이션</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>LLM 공급자·모델</t>
+          <t>인덱스·파티션·복제</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>솔버와 그 내부 표현</t>
+          <t>API endpoint</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>위험·신선도·근거 강도의 실제 임계값</t>
+          <t>LLM 공급자·모델</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>plan_decision.decision_type 의 값 목록</t>
+          <t>솔버와 그 내부 표현</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>applicability_scope_type 값 목록 (L-14)</t>
+          <t>위험·신선도·근거 강도의 실제 임계값</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>복구 맥락 식별자 (L-13)</t>
+          <t>plan_decision.decision_type 의 값 목록</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>bl 의 실제 UNIQUE 제약 (L-16)</t>
+          <t>applicability_scope_type 값 목록 (L-14)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>적용 범위 사이의 우선순위 규칙 (L-14)</t>
+          <t>복구 맥락 식별자 (L-13)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>system_error 오류 분류·코드 값 목록 (Q-66)</t>
+          <t>bl 의 실제 UNIQUE 제약 (L-16)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Backend 언어·프레임워크 (ADR-031 Proposed, docs/23)</t>
+          <t>적용 범위 사이의 우선순위 규칙 (L-14)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>event.idempotency_key 의 직렬화·해시 알고리즘·주장 위치(claim locator) 형식 (11.2d)</t>
+          <t>system_error 오류 분류·코드 값 목록 (Q-66)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>event.schema_version 문자열 형식</t>
+          <t>Backend 언어·프레임워크 (ADR-031 Proposed, docs/23)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
+          <t>event.idempotency_key 의 직렬화·해시 알고리즘·주장 위치(claim locator) 형식 (11.2d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>event.schema_version 문자열 형식</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
           <t>input_confidence_reasons / validator_result 의 JSON 구조 세부</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>실제 메일 보관 기간 숫자 (Q-45 기간 - Pilot 정책) / 보관 관리 내용의 물리 저장 위치</t>
         </is>
       </c>
     </row>
@@ -11469,7 +11541,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>rev.2: payload_hash UNIQUE 제거. 내용이 같아도 재수집은 새 관측이다 (예시 1·2 는 같은 해시). 중복 처리 차단은 출처가 주는 source_record_key 로만 한다 / rev.2.3: source_type 값을 ADR-020 7값으로 맞췄다 (event.source_type 과 같은 집합)</t>
+          <t>rev.2: payload_hash UNIQUE 제거. 내용이 같아도 재수집은 새 관측이다 (예시 1·2 는 같은 해시). 중복 처리 차단은 출처가 주는 source_record_key 로만 한다 / rev.2.3: source_type 값을 ADR-020 7값으로 맞췄다 (event.source_type 과 같은 집합) / rev.2.4 (Q-45): 원문은 보관 관리 내용. 보관 기간이 끝나면 원문만 파기되고 이 행·지문·외부 id·시각은 남는다. source_recorded_at 은 메일이면 Q-44 규칙(Date 가 채널 수신 시각보다 미래가 아니면 Date)</t>
         </is>
       </c>
     </row>
@@ -11511,25 +11583,30 @@
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
+          <t>첨부 목록</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
           <t>출처 전달 키</t>
         </is>
       </c>
-      <c r="I11" s="16" t="inlineStr">
+      <c r="J11" s="16" t="inlineStr">
         <is>
           <t>출처 기록 시각</t>
         </is>
       </c>
-      <c r="J11" s="16" t="inlineStr">
+      <c r="K11" s="16" t="inlineStr">
         <is>
           <t>수신 시각</t>
         </is>
       </c>
-      <c r="K11" s="16" t="inlineStr">
+      <c r="L11" s="16" t="inlineStr">
         <is>
           <t>수집 주체</t>
         </is>
       </c>
-      <c r="L11" s="16" t="inlineStr">
+      <c r="M11" s="16" t="inlineStr">
         <is>
           <t>시뮬레이션</t>
         </is>
@@ -11561,7 +11638,7 @@
           <t>request_ref</t>
         </is>
       </c>
-      <c r="F12" s="17" t="inlineStr">
+      <c r="F12" s="19" t="inlineStr">
         <is>
           <t>payload_ref</t>
         </is>
@@ -11571,27 +11648,32 @@
           <t>payload_hash</t>
         </is>
       </c>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>attachment_manifest</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
         <is>
           <t>source_record_key</t>
         </is>
       </c>
-      <c r="I12" s="17" t="inlineStr">
+      <c r="J12" s="17" t="inlineStr">
         <is>
           <t>source_recorded_at</t>
         </is>
       </c>
-      <c r="J12" s="17" t="inlineStr">
+      <c r="K12" s="17" t="inlineStr">
         <is>
           <t>received_at</t>
         </is>
       </c>
-      <c r="K12" s="17" t="inlineStr">
+      <c r="L12" s="17" t="inlineStr">
         <is>
           <t>collected_by_actor_id</t>
         </is>
       </c>
-      <c r="L12" s="17" t="inlineStr">
+      <c r="M12" s="17" t="inlineStr">
         <is>
           <t>is_simulated</t>
         </is>
@@ -11635,25 +11717,30 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
           <t>STRING(200)</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>TIMESTAMP_TZ</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>TIMESTAMP_TZ</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>REF(actor)</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
         </is>
@@ -11687,35 +11774,40 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
+          <t>NULL 허용 / 보관 관리 내용 참조(29절). 파기돼도 참조는 남는다 / rev.2.4</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL / UNIQUE 아님</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용 / 첨부마다 지문·크기·형식만. 파일명·내용 금지 / rev.2.4 신규</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>출처가 줄 때만 / 있을 때 유일</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
           <t>NULL 허용</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>NOT NULL / UNIQUE 아님</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>출처가 줄 때만 / 있을 때 유일</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>NULL 허용</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>NULL 허용</t>
-        </is>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
@@ -11747,33 +11839,30 @@
           <t>blYy=2026&amp;blNo=* (마스킹)</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>store://raw/000001</t>
-        </is>
-      </c>
+      <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="inlineStr">
         <is>
           <t>(해시값)</t>
         </is>
       </c>
       <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>2026-09-18T06:00+09:00</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>2026-09-18T06:00+09:00</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>ACT-SYS-01</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -11805,33 +11894,30 @@
           <t>blYy=2026&amp;blNo=* (마스킹)</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>store://raw/000003</t>
-        </is>
-      </c>
+      <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="inlineStr">
         <is>
           <t>(같은 해시값)</t>
         </is>
       </c>
       <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>2026-09-18T10:00+09:00</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>2026-09-18T10:00+09:00</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t>ACT-SYS-01</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -11859,37 +11945,34 @@
         </is>
       </c>
       <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>store://raw/000009</t>
-        </is>
-      </c>
+      <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="inlineStr">
         <is>
           <t>(해시값)</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>mock-msg-0021</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>2026-09-18T10:30+09:00</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>2026-09-18T10:30+09:00</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr">
         <is>
           <t>ACT-SYS-01</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -17491,7 +17574,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>계산에 들어가려면 사건이 되어 사실로 채택되어야 한다</t>
+          <t>계산에 들어가려면 사건이 되어 사실로 채택되어야 한다 / rev.2.4 (Q-45): 조건 원문은 보관 관리 내용. 계산에 쓰는 값은 commercial_offer_item</t>
         </is>
       </c>
     </row>
@@ -17548,20 +17631,25 @@
       </c>
       <c r="K30" s="16" t="inlineStr">
         <is>
-          <t>조건 원문</t>
+          <t>조건 원문 참조</t>
         </is>
       </c>
       <c r="L30" s="16" t="inlineStr">
         <is>
+          <t>조건 원문 지문</t>
+        </is>
+      </c>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
           <t>상태</t>
         </is>
       </c>
-      <c r="M30" s="16" t="inlineStr">
+      <c r="N30" s="16" t="inlineStr">
         <is>
           <t>시뮬레이션</t>
         </is>
       </c>
-      <c r="N30" s="16" t="inlineStr">
+      <c r="O30" s="16" t="inlineStr">
         <is>
           <t>시나리오</t>
         </is>
@@ -17620,20 +17708,25 @@
       </c>
       <c r="K31" s="19" t="inlineStr">
         <is>
-          <t>conditions_text</t>
+          <t>conditions_content_ref</t>
         </is>
       </c>
       <c r="L31" s="19" t="inlineStr">
         <is>
+          <t>conditions_hash</t>
+        </is>
+      </c>
+      <c r="M31" s="19" t="inlineStr">
+        <is>
           <t>offer_status</t>
         </is>
       </c>
-      <c r="M31" s="19" t="inlineStr">
+      <c r="N31" s="19" t="inlineStr">
         <is>
           <t>is_simulated</t>
         </is>
       </c>
-      <c r="N31" s="20" t="inlineStr">
+      <c r="O31" s="20" t="inlineStr">
         <is>
           <t>scenario_id</t>
         </is>
@@ -17692,20 +17785,25 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>STRING(300)</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr">
         <is>
+          <t>HASH</t>
+        </is>
+      </c>
+      <c r="M32" s="6" t="inlineStr">
+        <is>
           <t>CODE</t>
         </is>
       </c>
-      <c r="M32" s="6" t="inlineStr">
+      <c r="N32" s="6" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
         </is>
       </c>
-      <c r="N32" s="6" t="inlineStr">
+      <c r="O32" s="6" t="inlineStr">
         <is>
           <t>REF(scenario)</t>
         </is>
@@ -17764,20 +17862,25 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>NULL 허용</t>
+          <t>NULL 허용 / 보관 관리 내용 참조(29절). 파기돼도 참조는 남는다 / rev.2.4 (옛 conditions_text)</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
+          <t>참조가 있으면 NOT NULL / 파기돼도 남는다 / rev.2.4 신규</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
           <t>RECEIVED / SUPERSEDED / EXPIRED / WITHDRAWN</t>
         </is>
       </c>
-      <c r="M33" s="3" t="inlineStr">
+      <c r="N33" s="3" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="N33" s="3" t="inlineStr">
+      <c r="O33" s="3" t="inlineStr">
         <is>
           <t>NULL 허용</t>
         </is>
@@ -17809,7 +17912,7 @@
           <t>MSG-000021</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="n"/>
       <c r="G34" s="3" t="inlineStr">
         <is>
           <t>QI-0002</t>
@@ -17830,22 +17933,19 @@
           <t>2026-09-20T23:59+09:00</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>주말 반입 불가 (예시)</t>
-        </is>
-      </c>
-      <c r="L34" s="3" t="inlineStr">
+      <c r="K34" s="3" t="n"/>
+      <c r="L34" s="3" t="n"/>
+      <c r="M34" s="3" t="inlineStr">
         <is>
           <t>RECEIVED</t>
         </is>
       </c>
-      <c r="M34" s="3" t="inlineStr">
+      <c r="N34" s="3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="N34" s="3" t="inlineStr"/>
+      <c r="O34" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
@@ -25509,7 +25609,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>rev.2: message_kind 신규. CONTACT_VERIFICATION 은 업무 발송 승인의 예외지만 구조화 값·질문 연결을 가질 수 없고 감사는 남는다. 실제 메일 본문은 커밋하지 않는다 (docs/01 6절)</t>
+          <t>rev.2: message_kind 신규. CONTACT_VERIFICATION 은 업무 발송 승인의 예외지만 구조화 값·질문 연결을 가질 수 없고 감사는 남는다. 실제 메일 본문은 커밋하지 않는다 (docs/01 6절) / rev.2.4 (Q-45): 제목·본문은 보관 관리 내용. content_hash 는 파기돼도 남아 승인·발송 대조에 쓰인다. 원본 HTML 은 저장하지 않는다</t>
         </is>
       </c>
     </row>
@@ -25566,59 +25666,55 @@
       </c>
       <c r="K30" s="16" t="inlineStr">
         <is>
-          <t>제목</t>
+          <t>제목·본문 참조</t>
         </is>
       </c>
       <c r="L30" s="16" t="inlineStr">
         <is>
-          <t>본문</t>
+          <t>본문 지문</t>
         </is>
       </c>
       <c r="M30" s="16" t="inlineStr">
         <is>
-          <t>본문 지문</t>
+          <t>현재 상태</t>
         </is>
       </c>
       <c r="N30" s="16" t="inlineStr">
         <is>
-          <t>현재 상태</t>
+          <t>현재 승인</t>
         </is>
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>현재 승인</t>
+          <t>작성 주체</t>
         </is>
       </c>
       <c r="P30" s="16" t="inlineStr">
         <is>
-          <t>작성 주체</t>
+          <t>생성 시각</t>
         </is>
       </c>
       <c r="Q30" s="16" t="inlineStr">
         <is>
-          <t>생성 시각</t>
+          <t>발송 시각</t>
         </is>
       </c>
       <c r="R30" s="16" t="inlineStr">
         <is>
-          <t>발송 시각</t>
+          <t>수신 시각</t>
         </is>
       </c>
       <c r="S30" s="16" t="inlineStr">
         <is>
-          <t>수신 시각</t>
+          <t>시뮬레이션</t>
         </is>
       </c>
       <c r="T30" s="16" t="inlineStr">
         <is>
-          <t>시뮬레이션</t>
-        </is>
-      </c>
-      <c r="U30" s="16" t="inlineStr">
-        <is>
           <t>시나리오</t>
         </is>
       </c>
+      <c r="U30" s="16" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -25673,59 +25769,55 @@
       </c>
       <c r="K31" s="19" t="inlineStr">
         <is>
-          <t>subject</t>
+          <t>message_content_ref</t>
         </is>
       </c>
       <c r="L31" s="19" t="inlineStr">
         <is>
-          <t>body_text</t>
+          <t>content_hash</t>
         </is>
       </c>
       <c r="M31" s="19" t="inlineStr">
         <is>
-          <t>content_hash</t>
-        </is>
-      </c>
-      <c r="N31" s="19" t="inlineStr">
-        <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="O31" s="20" t="inlineStr">
+      <c r="N31" s="20" t="inlineStr">
         <is>
           <t>current_approval_id</t>
         </is>
       </c>
+      <c r="O31" s="19" t="inlineStr">
+        <is>
+          <t>drafted_by</t>
+        </is>
+      </c>
       <c r="P31" s="19" t="inlineStr">
         <is>
-          <t>drafted_by</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="Q31" s="19" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>sent_at</t>
         </is>
       </c>
       <c r="R31" s="19" t="inlineStr">
         <is>
-          <t>sent_at</t>
+          <t>received_at</t>
         </is>
       </c>
       <c r="S31" s="19" t="inlineStr">
         <is>
-          <t>received_at</t>
-        </is>
-      </c>
-      <c r="T31" s="19" t="inlineStr">
-        <is>
           <t>is_simulated</t>
         </is>
       </c>
-      <c r="U31" s="20" t="inlineStr">
+      <c r="T31" s="20" t="inlineStr">
         <is>
           <t>scenario_id</t>
         </is>
       </c>
+      <c r="U31" s="20" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -25785,27 +25877,27 @@
       </c>
       <c r="L32" s="6" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>HASH</t>
         </is>
       </c>
       <c r="M32" s="6" t="inlineStr">
         <is>
-          <t>HASH</t>
+          <t>CODE</t>
         </is>
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
+          <t>REF(message_approval)</t>
+        </is>
+      </c>
+      <c r="O32" s="6" t="inlineStr">
+        <is>
           <t>CODE</t>
         </is>
       </c>
-      <c r="O32" s="6" t="inlineStr">
-        <is>
-          <t>REF(message_approval)</t>
-        </is>
-      </c>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>CODE</t>
+          <t>TIMESTAMP_TZ</t>
         </is>
       </c>
       <c r="Q32" s="6" t="inlineStr">
@@ -25820,19 +25912,15 @@
       </c>
       <c r="S32" s="6" t="inlineStr">
         <is>
-          <t>TIMESTAMP_TZ</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="T32" s="6" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
-        </is>
-      </c>
-      <c r="U32" s="6" t="inlineStr">
-        <is>
           <t>REF(scenario)</t>
         </is>
       </c>
+      <c r="U32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -25887,59 +25975,55 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
+          <t>NULL 허용 / 제목 + 안전한 텍스트 본문 한 묶음. 보관 관리 내용 참조(29절). 파기돼도 참조는 남는다 / rev.2.4 (옛 subject · body_text)</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL / 수신자+제목+본문+구조화 값을 덮는다</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL / 캐시</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용 / 편의 포인터</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>AI_DRAFT / HUMAN / TEMPLATE</t>
+        </is>
+      </c>
+      <c r="P33" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
           <t>NULL 허용</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr">
-        <is>
-          <t>NULL 허용 / AI 는 문장만 쓴다</t>
-        </is>
-      </c>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>NOT NULL / 수신자+제목+본문+구조화 값을 덮는다</t>
-        </is>
-      </c>
-      <c r="N33" s="3" t="inlineStr">
-        <is>
-          <t>NOT NULL / 캐시</t>
-        </is>
-      </c>
-      <c r="O33" s="3" t="inlineStr">
-        <is>
-          <t>NULL 허용 / 편의 포인터</t>
-        </is>
-      </c>
-      <c r="P33" s="3" t="inlineStr">
-        <is>
-          <t>AI_DRAFT / HUMAN / TEMPLATE</t>
-        </is>
-      </c>
-      <c r="Q33" s="3" t="inlineStr">
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용</t>
+        </is>
+      </c>
+      <c r="S33" s="3" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="R33" s="3" t="inlineStr">
+      <c r="T33" s="3" t="inlineStr">
         <is>
           <t>NULL 허용</t>
         </is>
       </c>
-      <c r="S33" s="3" t="inlineStr">
-        <is>
-          <t>NULL 허용</t>
-        </is>
-      </c>
-      <c r="T33" s="3" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="U33" s="3" t="inlineStr">
-        <is>
-          <t>NULL 허용</t>
-        </is>
-      </c>
+      <c r="U33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="21" t="inlineStr">
@@ -25967,7 +26051,7 @@
           <t>BUSINESS</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="n"/>
       <c r="G34" s="3" t="inlineStr">
         <is>
           <t>MOCK</t>
@@ -25988,53 +26072,45 @@
           <t>AD-0002</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>9/18 입고 가능 수량 문의 (예시)</t>
-        </is>
-      </c>
+      <c r="K34" s="3" t="n"/>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>(본문 - 합성)</t>
+          <t>(해시값)</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>(해시값)</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="N34" s="3" t="inlineStr">
         <is>
-          <t>SENT</t>
+          <t>APV-0001</t>
         </is>
       </c>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>APV-0001</t>
+          <t>AI_DRAFT</t>
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr">
         <is>
-          <t>AI_DRAFT</t>
+          <t>2026-09-18T09:10+09:00</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>2026-09-18T09:10+09:00</t>
-        </is>
-      </c>
-      <c r="R34" s="3" t="inlineStr">
-        <is>
           <t>2026-09-18T09:12+09:00</t>
         </is>
       </c>
-      <c r="S34" s="3" t="inlineStr"/>
-      <c r="T34" s="3" t="inlineStr">
+      <c r="R34" s="3" t="n"/>
+      <c r="S34" s="3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="U34" s="3" t="inlineStr"/>
+      <c r="T34" s="3" t="n"/>
+      <c r="U34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="21" t="inlineStr">
@@ -26062,7 +26138,7 @@
           <t>BUSINESS</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="n"/>
       <c r="G35" s="3" t="inlineStr">
         <is>
           <t>MOCK</t>
@@ -26078,50 +26154,42 @@
           <t>odcy@example.invalid</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr"/>
-      <c r="K35" s="3" t="inlineStr">
-        <is>
-          <t>RE: 요율 문의 (예시)</t>
-        </is>
-      </c>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>(본문 - 합성)</t>
+          <t>(해시값)</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>(해시값)</t>
-        </is>
-      </c>
-      <c r="N35" s="3" t="inlineStr">
-        <is>
           <t>REPLIED</t>
         </is>
       </c>
-      <c r="O35" s="3" t="inlineStr"/>
+      <c r="N35" s="3" t="n"/>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t>HUMAN</t>
+        </is>
+      </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>HUMAN</t>
-        </is>
-      </c>
-      <c r="Q35" s="3" t="inlineStr">
-        <is>
           <t>2026-09-18T10:30+09:00</t>
         </is>
       </c>
-      <c r="R35" s="3" t="inlineStr"/>
+      <c r="Q35" s="3" t="n"/>
+      <c r="R35" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T10:30+09:00</t>
+        </is>
+      </c>
       <c r="S35" s="3" t="inlineStr">
         <is>
-          <t>2026-09-18T10:30+09:00</t>
-        </is>
-      </c>
-      <c r="T35" s="3" t="inlineStr">
-        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="U35" s="3" t="inlineStr"/>
+      <c r="T35" s="3" t="n"/>
+      <c r="U35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="21" t="inlineStr">
@@ -26174,30 +26242,26 @@
           <t>AD-0001</t>
         </is>
       </c>
-      <c r="K36" s="3" t="inlineStr">
-        <is>
-          <t>주소 확인 안내 (예시)</t>
-        </is>
-      </c>
+      <c r="K36" s="3" t="n"/>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>(토큰 링크만 - 합성)</t>
+          <t>(해시값)</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
         <is>
-          <t>(해시값)</t>
-        </is>
-      </c>
-      <c r="N36" s="3" t="inlineStr">
-        <is>
           <t>SENT</t>
         </is>
       </c>
-      <c r="O36" s="3" t="inlineStr"/>
+      <c r="N36" s="3" t="n"/>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>TEMPLATE</t>
+        </is>
+      </c>
       <c r="P36" s="3" t="inlineStr">
         <is>
-          <t>TEMPLATE</t>
+          <t>2026-09-16T09:50+09:00</t>
         </is>
       </c>
       <c r="Q36" s="3" t="inlineStr">
@@ -26205,18 +26269,14 @@
           <t>2026-09-16T09:50+09:00</t>
         </is>
       </c>
-      <c r="R36" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-16T09:50+09:00</t>
-        </is>
-      </c>
-      <c r="S36" s="3" t="inlineStr"/>
-      <c r="T36" s="3" t="inlineStr">
+      <c r="R36" s="3" t="n"/>
+      <c r="S36" s="3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="U36" s="3" t="inlineStr"/>
+      <c r="T36" s="3" t="n"/>
+      <c r="U36" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
@@ -26806,7 +26866,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>rev.2.1·rev.2.2: 행 종류별 필수 컬럼이 다르다. APPROVED = approved_content_hash · approved_to_address_id 필수 + 메시지에 값이 있는 범위에서 제목·본문·구조화 값 사본 필수. REJECTED/REVISION_REQUESTED = reason 필수, 사본 조건을 적용하지 않는다. REVOKED/INVALIDATED = invalidates_approval_id + invalidation_cause 필수, 새 지문·사본 불필요, 대상은 같은 message_id 의 기존 APPROVED. 만료는 expires_at(만들 때 정함). 어떤 행도 UPDATE 하지 않는다</t>
+          <t>rev.2.1·rev.2.2: 행 종류별 필수 컬럼이 다르다. APPROVED = approved_content_hash · approved_to_address_id 필수 + 메시지에 값이 있는 범위에서 제목·본문·구조화 값 사본 필수. REJECTED/REVISION_REQUESTED = reason 필수, 사본 조건을 적용하지 않는다. REVOKED/INVALIDATED = invalidates_approval_id + invalidation_cause 필수, 새 지문·사본 불필요, 대상은 같은 message_id 의 기존 APPROVED. 만료는 expires_at(만들 때 정함). 어떤 행도 UPDATE 하지 않는다 / rev.2.4 (Q-45): 승인 문장 사본은 보관 관리 내용. approved_content_hash 와 승인·무효화 사슬은 기록으로 남는다. 유효한 승인의 사본은 파기하지 않는다</t>
         </is>
       </c>
     </row>
@@ -26858,34 +26918,30 @@
       </c>
       <c r="J60" s="16" t="inlineStr">
         <is>
-          <t>승인 시점 제목</t>
+          <t>승인 제목·본문 참조</t>
         </is>
       </c>
       <c r="K60" s="16" t="inlineStr">
         <is>
-          <t>승인 시점 본문</t>
+          <t>승인 시점 계획</t>
         </is>
       </c>
       <c r="L60" s="16" t="inlineStr">
         <is>
-          <t>승인 시점 계획</t>
+          <t>승인 내용 지문</t>
         </is>
       </c>
       <c r="M60" s="16" t="inlineStr">
         <is>
-          <t>승인 내용 지문</t>
+          <t>승인 시점 수신자</t>
         </is>
       </c>
       <c r="N60" s="16" t="inlineStr">
         <is>
-          <t>승인 시점 수신자</t>
-        </is>
-      </c>
-      <c r="O60" s="16" t="inlineStr">
-        <is>
           <t>사유</t>
         </is>
       </c>
+      <c r="O60" s="16" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -26935,34 +26991,30 @@
       </c>
       <c r="J61" s="19" t="inlineStr">
         <is>
-          <t>approved_subject</t>
-        </is>
-      </c>
-      <c r="K61" s="19" t="inlineStr">
-        <is>
-          <t>approved_body_text</t>
-        </is>
-      </c>
-      <c r="L61" s="20" t="inlineStr">
+          <t>approved_content_ref</t>
+        </is>
+      </c>
+      <c r="K61" s="20" t="inlineStr">
         <is>
           <t>approved_plan_run_id</t>
         </is>
       </c>
-      <c r="M61" s="19" t="inlineStr">
+      <c r="L61" s="19" t="inlineStr">
         <is>
           <t>approved_content_hash</t>
         </is>
       </c>
-      <c r="N61" s="20" t="inlineStr">
+      <c r="M61" s="20" t="inlineStr">
         <is>
           <t>approved_to_address_id</t>
         </is>
       </c>
-      <c r="O61" s="19" t="inlineStr">
+      <c r="N61" s="19" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
       </c>
+      <c r="O61" s="19" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -27017,29 +27069,25 @@
       </c>
       <c r="K62" s="6" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>REF(recovery_run)</t>
         </is>
       </c>
       <c r="L62" s="6" t="inlineStr">
         <is>
-          <t>REF(recovery_run)</t>
+          <t>HASH</t>
         </is>
       </c>
       <c r="M62" s="6" t="inlineStr">
         <is>
-          <t>HASH</t>
+          <t>REF(contact_channel_address)</t>
         </is>
       </c>
       <c r="N62" s="6" t="inlineStr">
         <is>
-          <t>REF(contact_channel_address)</t>
-        </is>
-      </c>
-      <c r="O62" s="6" t="inlineStr">
-        <is>
           <t>STRING(500)</t>
         </is>
       </c>
+      <c r="O62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -27089,34 +27137,30 @@
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>APPROVED 이고 원 메시지에 값이 있으면 필수 / 사본 (값이 없는 메시지에 빈 사본을 요구하지 않는다)</t>
+          <t>조건부 - APPROVED 이고 메시지에 제목·본문이 있으면 NOT NULL / 보관 관리 내용 참조(29절). 파기돼도 참조는 남는다 / rev.2.4</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>APPROVED 이고 원 메시지에 값이 있으면 필수 / 사본 (값이 없는 메시지에 빈 사본을 요구하지 않는다)</t>
+          <t>NULL 허용 / 계획 기반 메시지의 APPROVED 면 필수</t>
         </is>
       </c>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t>NULL 허용 / 계획 기반 메시지의 APPROVED 면 필수</t>
+          <t>APPROVED 면 필수 / REVOKED·INVALIDATED 는 불필요 / 구조화 값까지 덮는다</t>
         </is>
       </c>
       <c r="M63" s="3" t="inlineStr">
         <is>
-          <t>APPROVED 면 필수 / REVOKED·INVALIDATED 는 불필요 / 구조화 값까지 덮는다</t>
+          <t>APPROVED 면 필수</t>
         </is>
       </c>
       <c r="N63" s="3" t="inlineStr">
         <is>
-          <t>APPROVED 면 필수</t>
-        </is>
-      </c>
-      <c r="O63" s="3" t="inlineStr">
-        <is>
           <t>REJECTED·REVISION_REQUESTED 면 필수 / 무효화일 때 권장</t>
         </is>
       </c>
+      <c r="O63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="21" t="inlineStr">
@@ -27139,8 +27183,8 @@
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr"/>
-      <c r="F64" s="3" t="inlineStr"/>
+      <c r="E64" s="3" t="n"/>
+      <c r="F64" s="3" t="n"/>
       <c r="G64" s="3" t="inlineStr">
         <is>
           <t>ACT-USR-01</t>
@@ -27156,32 +27200,24 @@
           <t>2026-09-18T17:00+09:00</t>
         </is>
       </c>
-      <c r="J64" s="3" t="inlineStr">
-        <is>
-          <t>9/18 입고 가능 수량 문의 (예시)</t>
-        </is>
-      </c>
+      <c r="J64" s="3" t="n"/>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>(승인 당시 본문 - 합성)</t>
+          <t>RUN-0001</t>
         </is>
       </c>
       <c r="L64" s="3" t="inlineStr">
         <is>
-          <t>RUN-0001</t>
+          <t>(해시값)</t>
         </is>
       </c>
       <c r="M64" s="3" t="inlineStr">
         <is>
-          <t>(해시값)</t>
-        </is>
-      </c>
-      <c r="N64" s="3" t="inlineStr">
-        <is>
           <t>AD-0002</t>
         </is>
       </c>
-      <c r="O64" s="3" t="inlineStr"/>
+      <c r="N64" s="3" t="n"/>
+      <c r="O64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="21" t="inlineStr">
@@ -27224,25 +27260,25 @@
           <t>2026-09-18T10:21+09:00</t>
         </is>
       </c>
-      <c r="I65" s="3" t="inlineStr"/>
-      <c r="J65" s="3" t="inlineStr"/>
-      <c r="K65" s="3" t="inlineStr"/>
+      <c r="I65" s="3" t="n"/>
+      <c r="J65" s="3" t="n"/>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>RUN-0002</t>
+        </is>
+      </c>
       <c r="L65" s="3" t="inlineStr">
         <is>
-          <t>RUN-0002</t>
-        </is>
-      </c>
-      <c r="M65" s="3" t="inlineStr">
-        <is>
           <t>(해시값)</t>
         </is>
       </c>
-      <c r="N65" s="3" t="inlineStr"/>
-      <c r="O65" s="3" t="inlineStr">
+      <c r="M65" s="3" t="n"/>
+      <c r="N65" s="3" t="inlineStr">
         <is>
           <t>계획이 RUN-0002 로 교체됨 (예시)</t>
         </is>
       </c>
+      <c r="O65" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
@@ -28538,7 +28574,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>rev.2.2: 추출 결과(후보 값·인용·모델 판·프롬프트 판 등)는 불변. 검토 4컬럼(review_status·reviewed_by_actor_id·reviewed_at·created_event_id)만 PENDING -&gt; ACCEPTED/REJECTED/SUPERSEDED 한 방향 한 번. 신원·권한·근거 강도·상태 확정·숫자는 여기서 정하지 않는다 (ADR-026·029) / rev.2.3: docs/21 13절이 요구하는 스키마 판·입력 해시·검증기 결과를 보강했다. 불변 컬럼 12 -&gt; 15 (Markdown 15.9.2)</t>
+          <t>rev.2.2: 추출 결과(후보 값·인용·모델 판·프롬프트 판 등)는 불변. 검토 4컬럼(review_status·reviewed_by_actor_id·reviewed_at·created_event_id)만 PENDING -&gt; ACCEPTED/REJECTED/SUPERSEDED 한 방향 한 번. 신원·권한·근거 강도·상태 확정·숫자는 여기서 정하지 않는다 (ADR-026·029) / rev.2.3: docs/21 13절이 요구하는 스키마 판·입력 해시·검증기 결과를 보강했다. 불변 컬럼 12 -&gt; 15 (Markdown 15.9.2) / rev.2.4 (Q-45): 인용은 원문의 일부라 보관 관리 내용(원문보다 오래 둘 수 있다). 불변 컬럼 16. PENDING 이거나 열린 확인 요청의 근거면 파기하지 않는다</t>
         </is>
       </c>
     </row>
@@ -28580,65 +28616,70 @@
       </c>
       <c r="H100" s="16" t="inlineStr">
         <is>
-          <t>근거 인용</t>
+          <t>근거 인용 참조</t>
         </is>
       </c>
       <c r="I100" s="16" t="inlineStr">
         <is>
+          <t>근거 인용 지문</t>
+        </is>
+      </c>
+      <c r="J100" s="16" t="inlineStr">
+        <is>
           <t>인용 위치</t>
         </is>
       </c>
-      <c r="J100" s="16" t="inlineStr">
+      <c r="K100" s="16" t="inlineStr">
         <is>
           <t>모델 판</t>
         </is>
       </c>
-      <c r="K100" s="16" t="inlineStr">
+      <c r="L100" s="16" t="inlineStr">
         <is>
           <t>프롬프트 판</t>
         </is>
       </c>
-      <c r="L100" s="16" t="inlineStr">
+      <c r="M100" s="16" t="inlineStr">
         <is>
           <t>모델 자기 점수</t>
         </is>
       </c>
-      <c r="M100" s="16" t="inlineStr">
+      <c r="N100" s="16" t="inlineStr">
         <is>
           <t>처리 상태</t>
         </is>
       </c>
-      <c r="N100" s="16" t="inlineStr">
+      <c r="O100" s="16" t="inlineStr">
         <is>
           <t>채택 주체</t>
         </is>
       </c>
-      <c r="O100" s="16" t="inlineStr">
+      <c r="P100" s="16" t="inlineStr">
         <is>
           <t>채택 시각</t>
         </is>
       </c>
-      <c r="P100" s="16" t="inlineStr">
+      <c r="Q100" s="16" t="inlineStr">
         <is>
           <t>생성 사건</t>
         </is>
       </c>
-      <c r="Q100" s="16" t="inlineStr">
+      <c r="R100" s="16" t="inlineStr">
         <is>
           <t>시뮬레이션</t>
         </is>
       </c>
-      <c r="R100" s="16" t="inlineStr">
+      <c r="S100" s="16" t="inlineStr">
         <is>
           <t>추출 스키마 판</t>
         </is>
       </c>
-      <c r="S100" s="16" t="inlineStr">
+      <c r="T100" s="16" t="inlineStr">
         <is>
           <t>입력 지문</t>
         </is>
       </c>
-      <c r="T100" s="16" t="inlineStr">
+      <c r="U100" s="16" t="inlineStr">
         <is>
           <t>검증기 결과</t>
         </is>
@@ -28682,65 +28723,70 @@
       </c>
       <c r="H101" s="19" t="inlineStr">
         <is>
-          <t>source_quote</t>
+          <t>source_quote_ref</t>
         </is>
       </c>
       <c r="I101" s="19" t="inlineStr">
         <is>
+          <t>source_quote_hash</t>
+        </is>
+      </c>
+      <c r="J101" s="19" t="inlineStr">
+        <is>
           <t>quote_location</t>
         </is>
       </c>
-      <c r="J101" s="19" t="inlineStr">
+      <c r="K101" s="19" t="inlineStr">
         <is>
           <t>model_version</t>
         </is>
       </c>
-      <c r="K101" s="19" t="inlineStr">
+      <c r="L101" s="19" t="inlineStr">
         <is>
           <t>prompt_version</t>
         </is>
       </c>
-      <c r="L101" s="19" t="inlineStr">
+      <c r="M101" s="19" t="inlineStr">
         <is>
           <t>model_confidence</t>
         </is>
       </c>
-      <c r="M101" s="19" t="inlineStr">
+      <c r="N101" s="19" t="inlineStr">
         <is>
           <t>review_status</t>
         </is>
       </c>
-      <c r="N101" s="20" t="inlineStr">
+      <c r="O101" s="20" t="inlineStr">
         <is>
           <t>reviewed_by_actor_id</t>
         </is>
       </c>
-      <c r="O101" s="19" t="inlineStr">
+      <c r="P101" s="19" t="inlineStr">
         <is>
           <t>reviewed_at</t>
         </is>
       </c>
-      <c r="P101" s="20" t="inlineStr">
+      <c r="Q101" s="20" t="inlineStr">
         <is>
           <t>created_event_id</t>
         </is>
       </c>
-      <c r="Q101" s="19" t="inlineStr">
+      <c r="R101" s="19" t="inlineStr">
         <is>
           <t>is_simulated</t>
         </is>
       </c>
-      <c r="R101" s="19" t="inlineStr">
+      <c r="S101" s="19" t="inlineStr">
         <is>
           <t>schema_version</t>
         </is>
       </c>
-      <c r="S101" s="19" t="inlineStr">
+      <c r="T101" s="19" t="inlineStr">
         <is>
           <t>input_hash</t>
         </is>
       </c>
-      <c r="T101" s="19" t="inlineStr">
+      <c r="U101" s="19" t="inlineStr">
         <is>
           <t>validator_result</t>
         </is>
@@ -28784,65 +28830,70 @@
       </c>
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>STRING(300)</t>
         </is>
       </c>
       <c r="I102" s="6" t="inlineStr">
         <is>
+          <t>HASH</t>
+        </is>
+      </c>
+      <c r="J102" s="6" t="inlineStr">
+        <is>
           <t>STRING(100)</t>
         </is>
       </c>
-      <c r="J102" s="6" t="inlineStr">
+      <c r="K102" s="6" t="inlineStr">
         <is>
           <t>STRING(60)</t>
         </is>
       </c>
-      <c r="K102" s="6" t="inlineStr">
+      <c r="L102" s="6" t="inlineStr">
         <is>
           <t>STRING(20)</t>
         </is>
       </c>
-      <c r="L102" s="6" t="inlineStr">
+      <c r="M102" s="6" t="inlineStr">
         <is>
           <t>DECIMAL(5,4)</t>
         </is>
       </c>
-      <c r="M102" s="6" t="inlineStr">
+      <c r="N102" s="6" t="inlineStr">
         <is>
           <t>CODE</t>
         </is>
       </c>
-      <c r="N102" s="6" t="inlineStr">
+      <c r="O102" s="6" t="inlineStr">
         <is>
           <t>REF(actor)</t>
         </is>
       </c>
-      <c r="O102" s="6" t="inlineStr">
+      <c r="P102" s="6" t="inlineStr">
         <is>
           <t>TIMESTAMP_TZ</t>
         </is>
       </c>
-      <c r="P102" s="6" t="inlineStr">
+      <c r="Q102" s="6" t="inlineStr">
         <is>
           <t>REF(event)</t>
         </is>
       </c>
-      <c r="Q102" s="6" t="inlineStr">
+      <c r="R102" s="6" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
         </is>
       </c>
-      <c r="R102" s="6" t="inlineStr">
+      <c r="S102" s="6" t="inlineStr">
         <is>
           <t>STRING(20)</t>
         </is>
       </c>
-      <c r="S102" s="6" t="inlineStr">
+      <c r="T102" s="6" t="inlineStr">
         <is>
           <t>HASH</t>
         </is>
       </c>
-      <c r="T102" s="6" t="inlineStr">
+      <c r="U102" s="6" t="inlineStr">
         <is>
           <t>JSON</t>
         </is>
@@ -28886,65 +28937,70 @@
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
+          <t>NOT NULL / 보관 관리 내용 참조(29절). 파기돼도 참조는 남는다 / rev.2.4 (옛 source_quote)</t>
+        </is>
+      </c>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL / 인용이 파기돼도 남는다 / rev.2.4 신규</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용</t>
+        </is>
+      </c>
+      <c r="K103" s="3" t="inlineStr">
+        <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="I103" s="3" t="inlineStr">
+      <c r="L103" s="3" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="M103" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용 / 근거 강도 아님</t>
+        </is>
+      </c>
+      <c r="N103" s="3" t="inlineStr">
+        <is>
+          <t>PENDING / ACCEPTED / REJECTED / SUPERSEDED - 한 방향 한 번</t>
+        </is>
+      </c>
+      <c r="O103" s="3" t="inlineStr">
         <is>
           <t>NULL 허용</t>
         </is>
       </c>
-      <c r="J103" s="3" t="inlineStr">
+      <c r="P103" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용</t>
+        </is>
+      </c>
+      <c r="Q103" s="3" t="inlineStr">
+        <is>
+          <t>NULL 허용 / ACCEPTED 면 필수</t>
+        </is>
+      </c>
+      <c r="R103" s="3" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="K103" s="3" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="L103" s="3" t="inlineStr">
-        <is>
-          <t>NULL 허용 / 근거 강도 아님</t>
-        </is>
-      </c>
-      <c r="M103" s="3" t="inlineStr">
-        <is>
-          <t>PENDING / ACCEPTED / REJECTED / SUPERSEDED - 한 방향 한 번</t>
-        </is>
-      </c>
-      <c r="N103" s="3" t="inlineStr">
-        <is>
-          <t>NULL 허용</t>
-        </is>
-      </c>
-      <c r="O103" s="3" t="inlineStr">
-        <is>
-          <t>NULL 허용</t>
-        </is>
-      </c>
-      <c r="P103" s="3" t="inlineStr">
-        <is>
-          <t>NULL 허용 / ACCEPTED 면 필수</t>
-        </is>
-      </c>
-      <c r="Q103" s="3" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="R103" s="3" t="inlineStr">
+      <c r="S103" s="3" t="inlineStr">
         <is>
           <t>NOT NULL / 어느 추출 계약으로 뽑았나 / rev.2.3 신규</t>
         </is>
       </c>
-      <c r="S103" s="3" t="inlineStr">
+      <c r="T103" s="3" t="inlineStr">
         <is>
           <t>NOT NULL / 무엇을 넣고 뽑았나 / rev.2.3 신규</t>
         </is>
       </c>
-      <c r="T103" s="3" t="inlineStr">
+      <c r="U103" s="3" t="inlineStr">
         <is>
           <t>NOT NULL / docs/05 4.6 검사별 결과 / model_confidence 와 다르다 / rev.2.3 신규</t>
         </is>
@@ -28986,67 +29042,64 @@
           <t>KRW</t>
         </is>
       </c>
-      <c r="H104" s="3" t="inlineStr">
-        <is>
-          <t>40피트 1회 95,000원입니다 (합성)</t>
-        </is>
-      </c>
-      <c r="I104" s="3" t="inlineStr">
+      <c r="H104" s="3" t="n"/>
+      <c r="I104" s="3" t="n"/>
+      <c r="J104" s="3" t="inlineStr">
         <is>
           <t>body:3</t>
         </is>
       </c>
-      <c r="J104" s="3" t="inlineStr">
+      <c r="K104" s="3" t="inlineStr">
         <is>
           <t>(모델 판)</t>
         </is>
       </c>
-      <c r="K104" s="3" t="inlineStr">
+      <c r="L104" s="3" t="inlineStr">
         <is>
           <t>p-v1</t>
         </is>
       </c>
-      <c r="L104" s="3" t="inlineStr">
+      <c r="M104" s="3" t="inlineStr">
         <is>
           <t>0.8800</t>
         </is>
       </c>
-      <c r="M104" s="3" t="inlineStr">
+      <c r="N104" s="3" t="inlineStr">
         <is>
           <t>ACCEPTED</t>
         </is>
       </c>
-      <c r="N104" s="3" t="inlineStr">
+      <c r="O104" s="3" t="inlineStr">
         <is>
           <t>ACT-USR-01</t>
         </is>
       </c>
-      <c r="O104" s="3" t="inlineStr">
+      <c r="P104" s="3" t="inlineStr">
         <is>
           <t>2026-09-18T10:40+09:00</t>
         </is>
       </c>
-      <c r="P104" s="3" t="inlineStr">
+      <c r="Q104" s="3" t="inlineStr">
         <is>
           <t>EVT-000061</t>
         </is>
       </c>
-      <c r="Q104" s="3" t="inlineStr">
+      <c r="R104" s="3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="R104" s="3" t="inlineStr">
+      <c r="S104" s="3" t="inlineStr">
         <is>
           <t>ex-1</t>
         </is>
       </c>
-      <c r="S104" s="3" t="inlineStr">
+      <c r="T104" s="3" t="inlineStr">
         <is>
           <t>(해시값)</t>
         </is>
       </c>
-      <c r="T104" s="3" t="inlineStr">
+      <c r="U104" s="3" t="inlineStr">
         <is>
           <t>[SCHEMA_OK, QUOTE_MATCHED]</t>
         </is>

</xml_diff>

<commit_message>
docs: finalize CERA external communication implementation plan
T-069 DONE. 첫 실제 구현 Vertical Slice 의 범위·순서·검증 기준을
docs/tasks/plans/T-069-external-communication-slice.md 로 확정한다.
제품 코드 없음. docs/21 변경 없음.

- Slice 1 = Mock External Communication Loop (docs/18 J.4 1·2단계)
  Slice 2 Tech Validation(등록·확인 메일·Gmail), Slice 3 실제 LLM
- L-13 CLOSED: 복구 맥락 = recovery_run 계보의 뿌리 실행 id
  (docs/22 I-35·I-36, 새 표·컬럼 없음)
- P0 29 · P1 14 · DEFERRED 9, Phase 0~11, DoD 19항목
- 정상 회신은 검증 통과 값이 사건 → PROVISIONAL → 사람 확인 →
  CONFIRMED. 사건 생성 승인 게이트 없음
- 지난 계획 기준 회신은 사건·후보가 되지만 현재 계획에 자동 반영되지
  않는다(계획 불변 · 자동 재최적화 없음 · 스레드 안 질문 매핑)
- DB 선택을 Q-68 로 등록. QUEUE: T-083(Q-64)·T-084(Q-68)
  NEEDS_HUMAN → T-080 → T-085~T-096(U0~U11). T-003 은 U0 에 흡수
- docs/18 N.2 #13 K.2 성공 판정 수 13 → 12 정정
</commit_message>
<xml_diff>
--- a/docs/22_cera-logical-data-model.xlsx
+++ b/docs/22_cera-logical-data-model.xlsx
@@ -3707,7 +3707,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="8" t="n">
         <v>2</v>
@@ -5135,6 +5134,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -5430,6 +5430,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
@@ -5533,6 +5534,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
@@ -6015,12 +6017,12 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>OPEN - rev.2 신규</t>
+          <t>CLOSED - T-069 (2026-09-21)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>후보: recovery_run 계보의 뿌리 / 최초 계기 사건 / 컨테이너 집합 지문. T-069 에서 답한다</t>
+          <t>recovery_run 계보(previous_run_id)의 뿌리 실행 id. 새 표·새 컬럼 없음. 같은 사고의 재계산은 previous_run_id 를 이어받는다. 범위 참조는 존재하는 뿌리 실행 id (I-35·I-36). ExceptionCase 부활 없음</t>
         </is>
       </c>
     </row>
@@ -6156,6 +6158,8 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="23" t="inlineStr">
         <is>
@@ -6236,7 +6240,7 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>복구 맥락 식별자 (L-13)</t>
+          <t>(닫힘) 복구 맥락 식별자 (L-13) — 2026-09-21 T-069 CLOSED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: finalize CERA P0 physical data model
</commit_message>
<xml_diff>
--- a/docs/22_cera-logical-data-model.xlsx
+++ b/docs/22_cera-logical-data-model.xlsx
@@ -581,7 +581,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>rev.2.4 Q-44 · Q-45 사용자 결정 반영 (2026-09-21). 메일 근거 시각 규칙 + 기록·내용 분리 보관. 표 수 변화 없음. 흐름 검증 64개 PASS. (rev.2.3 T-081 DONE 위)</t>
+          <t>rev.2.5 T-080 물리 설계 검토 반영 (2026-09-22). 발송 시도 멱등·재시도·UNKNOWN 화해 · sent_at / external_thread_id 한 번 채움 · INBOUND drafted_by·current_status · 표기 정정. 표·컬럼 수 변화 없음. (rev.2.4 Q-44 · Q-45 위)</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>CONTROLLED_UPDATE (thread_status · last_activity_at)</t>
+          <t>CONTROLLED_UPDATE (thread_status · last_activity_at) + external_thread_id 한 번 채움</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>IMMUTABLE_AFTER_CREATE + CACHE_UPDATE</t>
+          <t>IMMUTABLE_AFTER_CREATE + CACHE_UPDATE + sent_at 한 번 채움</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>IMMUTABLE_AFTER_CREATE + CONTROLLED_UPDATE (결과 5컬럼)</t>
+          <t>IMMUTABLE_AFTER_CREATE + CONTROLLED_UPDATE (결과 5컬럼 · UNKNOWN 화해 한 번)</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -5134,7 +5134,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -5430,7 +5429,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
@@ -5534,7 +5532,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
@@ -6158,8 +6155,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50"/>
     <row r="51">
       <c r="A51" s="23" t="inlineStr">
         <is>
@@ -13466,7 +13461,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>SUBJECT / CONTEXT</t>
+          <t>NOT NULL / SUBJECT / CONTEXT (rev.2.5 표기 정정 — I-8)</t>
         </is>
       </c>
     </row>
@@ -14500,7 +14495,7 @@
       </c>
       <c r="W57" s="3" t="inlineStr">
         <is>
-          <t>NOT NULL / 계산 결과</t>
+          <t>NOT NULL / 계산 결과 / 강도 0·1·2·3 (docs/05 3.3, rev.2.5)</t>
         </is>
       </c>
       <c r="X57" s="3" t="inlineStr">
@@ -14646,7 +14641,7 @@
       </c>
       <c r="W58" s="3" t="inlineStr">
         <is>
-          <t>STRONG</t>
+          <t>3</t>
         </is>
       </c>
       <c r="X58" s="3" t="inlineStr">
@@ -14661,7 +14656,7 @@
       </c>
       <c r="Z58" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_EVENT_TIME</t>
+          <t>EVENT_TIME</t>
         </is>
       </c>
       <c r="AA58" s="3" t="inlineStr">
@@ -14796,7 +14791,7 @@
       </c>
       <c r="W59" s="3" t="inlineStr">
         <is>
-          <t>STRONG</t>
+          <t>3</t>
         </is>
       </c>
       <c r="X59" s="3" t="inlineStr">
@@ -14811,7 +14806,7 @@
       </c>
       <c r="Z59" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_EVENT_TIME</t>
+          <t>EVENT_TIME</t>
         </is>
       </c>
       <c r="AA59" s="3" t="inlineStr">
@@ -24554,7 +24549,7 @@
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>CONTROLLED_UPDATE (thread_status · last_activity_at)</t>
+          <t>CONTROLLED_UPDATE (thread_status · last_activity_at) + external_thread_id 한 번 채움</t>
         </is>
       </c>
     </row>
@@ -24789,7 +24784,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>NULL 허용</t>
+          <t>NULL 허용 / 첫 발송 뒤 NULL → 값 한 번(rev.2.5)</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -24901,6 +24896,7 @@
       </c>
       <c r="M14" s="3" t="inlineStr"/>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="n">
         <v>2</v>
@@ -25538,6 +25534,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="8" t="n">
         <v>3</v>
@@ -25589,7 +25586,7 @@
       </c>
       <c r="K27" s="9" t="inlineStr">
         <is>
-          <t>IMMUTABLE_AFTER_CREATE + CACHE_UPDATE</t>
+          <t>IMMUTABLE_AFTER_CREATE + CACHE_UPDATE + sent_at 한 번 채움</t>
         </is>
       </c>
     </row>
@@ -25989,7 +25986,7 @@
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>NOT NULL / 캐시</t>
+          <t>OUTBOUND 면 NOT NULL / 캐시 / INBOUND 는 NULL(rev.2.5)</t>
         </is>
       </c>
       <c r="N33" s="3" t="inlineStr">
@@ -25999,7 +25996,7 @@
       </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>AI_DRAFT / HUMAN / TEMPLATE</t>
+          <t>OUTBOUND 면 필수 / AI_DRAFT / HUMAN / TEMPLATE / INBOUND 는 NULL(rev.2.5)</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
@@ -26009,7 +26006,7 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>NULL 허용</t>
+          <t>NULL 허용 / 발송 성공 확인 뒤 NULL → 값 한 번(rev.2.5)</t>
         </is>
       </c>
       <c r="R33" s="3" t="inlineStr">
@@ -26282,6 +26279,7 @@
       <c r="T36" s="3" t="n"/>
       <c r="U36" s="3" t="n"/>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="8" t="n">
         <v>4</v>
@@ -26631,6 +26629,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="8" t="n">
         <v>5</v>
@@ -26795,6 +26794,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="8" t="n">
         <v>6</v>
@@ -27284,6 +27284,7 @@
       </c>
       <c r="O65" s="3" t="n"/>
     </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" s="8" t="n">
         <v>7</v>
@@ -27633,6 +27634,7 @@
         </is>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="8" t="n">
         <v>8</v>
@@ -27684,7 +27686,7 @@
       </c>
       <c r="K77" s="9" t="inlineStr">
         <is>
-          <t>IMMUTABLE_AFTER_CREATE + CONTROLLED_UPDATE (결과 5컬럼)</t>
+          <t>IMMUTABLE_AFTER_CREATE + CONTROLLED_UPDATE (결과 5컬럼 · UNKNOWN 화해 한 번)</t>
         </is>
       </c>
     </row>
@@ -27971,7 +27973,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>NOT NULL / 채널+메시지+내용지문+(있으면)승인</t>
+          <t>NOT NULL / UNIQUE / 시도마다 다름: 메시지 + 시도 번호(rev.2.5)</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -27996,7 +27998,7 @@
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>NULL = 결과 기록 전 / SUCCESS / RETRYABLE_FAILURE / PERMANENT_FAILURE / UNKNOWN - 한 번만</t>
+          <t>NULL = 결과 기록 전 / SUCCESS / RETRYABLE_FAILURE / PERMANENT_FAILURE / UNKNOWN - NULL → 결과 한 번, UNKNOWN 은 화해로 SUCCESS · RETRYABLE_FAILURE 한 번 더(rev.2.5)</t>
         </is>
       </c>
       <c r="L83" s="3" t="inlineStr">
@@ -28048,7 +28050,7 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>MOCK:MSG-000020:(해시값):APV-0001</t>
+          <t>(해시: MSG-000020 · 시도 1)</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -28113,7 +28115,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>MOCK:MSG-000030:(해시값)</t>
+          <t>(해시: MSG-000030 · 시도 1)</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -28154,6 +28156,7 @@
         </is>
       </c>
     </row>
+    <row r="86"/>
     <row r="87">
       <c r="A87" s="8" t="n">
         <v>9</v>
@@ -28503,6 +28506,7 @@
         </is>
       </c>
     </row>
+    <row r="96"/>
     <row r="97">
       <c r="A97" s="8" t="n">
         <v>10</v>

</xml_diff>